<commit_message>
Cek 1: kode E1 untuk idx 1338; Cek 2: buat ulang lembar mengikuti korpus terkini (C1 195, C3 176, eksklusi 143)
Claude-Session: https://claude.ai/code/session_01WzxXUNuhBFZJ8eSS7mVYXf
</commit_message>
<xml_diff>
--- a/literature/scopus-2026-09/verifikasi/cek-2-cek-tangan/cek_C3.xlsx
+++ b/literature/scopus-2026-09/verifikasi/cek-2-cek-tangan/cek_C3.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="keterangan" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'cek'!$A$1:$T$171</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'cek'!$A$1:$T$177</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T171"/>
+  <dimension ref="A1:T177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -782,7 +782,7 @@
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
@@ -840,12 +840,12 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>KLS</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>TANAH</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -881,11 +881,7 @@
       <c r="Q5" s="5" t="inlineStr"/>
       <c r="R5" s="5" t="inlineStr"/>
       <c r="S5" s="6" t="inlineStr"/>
-      <c r="T5" s="4" t="inlineStr">
-        <is>
-          <t>kode '?' pada: lokasi</t>
-        </is>
-      </c>
+      <c r="T5" s="4" t="inlineStr"/>
     </row>
     <row r="6" ht="110" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1312,7 +1308,7 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>KLS</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
@@ -1493,10 +1489,14 @@
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O13" s="3" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/narendran2024palm.txt</t>
+        </is>
+      </c>
       <c r="P13" s="3" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1507,7 +1507,7 @@
       <c r="S13" s="6" t="inlineStr"/>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
+          <t>kode '?' pada: lokasi</t>
         </is>
       </c>
     </row>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>POHON</t>
+          <t>TANAH</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
@@ -1713,20 +1713,24 @@
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="N16" s="3" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O16" s="3" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/daud2023detection.txt</t>
+        </is>
+      </c>
       <c r="P16" s="3" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1735,11 +1739,7 @@
       <c r="Q16" s="5" t="inlineStr"/>
       <c r="R16" s="5" t="inlineStr"/>
       <c r="S16" s="6" t="inlineStr"/>
-      <c r="T16" s="4" t="inlineStr">
-        <is>
-          <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI</t>
-        </is>
-      </c>
+      <c r="T16" s="4" t="inlineStr"/>
     </row>
     <row r="17" ht="110" customHeight="1">
       <c r="A17" s="3" t="n">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
@@ -2499,10 +2499,14 @@
       </c>
       <c r="N26" s="3" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O26" s="3" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O26" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/prasetyo2020automatic.txt</t>
+        </is>
+      </c>
       <c r="P26" s="3" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2511,11 +2515,7 @@
       <c r="Q26" s="5" t="inlineStr"/>
       <c r="R26" s="5" t="inlineStr"/>
       <c r="S26" s="6" t="inlineStr"/>
-      <c r="T26" s="4" t="inlineStr">
-        <is>
-          <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI</t>
-        </is>
-      </c>
+      <c r="T26" s="4" t="inlineStr"/>
     </row>
     <row r="27" ht="110" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -2646,7 +2646,7 @@
       </c>
       <c r="M28" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="N28" s="3" t="inlineStr">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>PABRIK</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
@@ -2743,7 +2743,7 @@
       <c r="S29" s="6" t="inlineStr"/>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
+          <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI</t>
         </is>
       </c>
     </row>
@@ -3114,7 +3114,7 @@
       </c>
       <c r="M34" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="N34" s="3" t="inlineStr">
@@ -3168,7 +3168,7 @@
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>KLS</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
@@ -3178,25 +3178,29 @@
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>RGB</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="N35" s="3" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O35" s="3" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O35" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/kassim2012oil.txt</t>
+        </is>
+      </c>
       <c r="P35" s="3" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3205,11 +3209,7 @@
       <c r="Q35" s="5" t="inlineStr"/>
       <c r="R35" s="5" t="inlineStr"/>
       <c r="S35" s="6" t="inlineStr"/>
-      <c r="T35" s="4" t="inlineStr">
-        <is>
-          <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: tugas, modalitas</t>
-        </is>
-      </c>
+      <c r="T35" s="4" t="inlineStr"/>
     </row>
     <row r="36" ht="110" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -3430,7 +3430,7 @@
       </c>
       <c r="M38" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="N38" s="3" t="inlineStr">
@@ -3676,15 +3676,19 @@
       </c>
       <c r="M41" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="N41" s="3" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O41" s="3" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O41" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/hamdani2026automated.txt</t>
+        </is>
+      </c>
       <c r="P41" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -3739,7 +3743,7 @@
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>PABRIK</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
@@ -3775,11 +3779,7 @@
       <c r="Q42" s="5" t="inlineStr"/>
       <c r="R42" s="5" t="inlineStr"/>
       <c r="S42" s="6" t="inlineStr"/>
-      <c r="T42" s="4" t="inlineStr">
-        <is>
-          <t>kode '?' pada: lokasi</t>
-        </is>
-      </c>
+      <c r="T42" s="4" t="inlineStr"/>
     </row>
     <row r="43" ht="110" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -3820,7 +3820,7 @@
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>MUTU</t>
+          <t>KLS</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
@@ -4080,7 +4080,7 @@
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>PABRIK</t>
         </is>
       </c>
       <c r="K46" s="3" t="inlineStr">
@@ -4116,11 +4116,7 @@
       <c r="Q46" s="5" t="inlineStr"/>
       <c r="R46" s="5" t="inlineStr"/>
       <c r="S46" s="6" t="inlineStr"/>
-      <c r="T46" s="4" t="inlineStr">
-        <is>
-          <t>kode '?' pada: lokasi</t>
-        </is>
-      </c>
+      <c r="T46" s="4" t="inlineStr"/>
     </row>
     <row r="47" ht="110" customHeight="1">
       <c r="A47" s="3" t="n">
@@ -4166,7 +4162,7 @@
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>POHON</t>
+          <t>PABRIK</t>
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr">
@@ -4249,7 +4245,7 @@
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>RGB+NIR</t>
+          <t>RGB</t>
         </is>
       </c>
       <c r="L48" s="3" t="inlineStr">
@@ -4330,7 +4326,7 @@
       </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
-          <t>POHON</t>
+          <t>?</t>
         </is>
       </c>
       <c r="K49" s="3" t="inlineStr">
@@ -4366,7 +4362,11 @@
       <c r="Q49" s="5" t="inlineStr"/>
       <c r="R49" s="5" t="inlineStr"/>
       <c r="S49" s="6" t="inlineStr"/>
-      <c r="T49" s="4" t="inlineStr"/>
+      <c r="T49" s="4" t="inlineStr">
+        <is>
+          <t>kode '?' pada: lokasi</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="110" customHeight="1">
       <c r="A50" s="3" t="n">
@@ -5312,7 +5312,7 @@
       </c>
       <c r="L61" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="M61" s="3" t="inlineStr">
@@ -5712,7 +5712,7 @@
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>POHON</t>
         </is>
       </c>
       <c r="K66" s="3" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="M66" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="N66" s="3" t="inlineStr">
@@ -5748,11 +5748,7 @@
       <c r="Q66" s="5" t="inlineStr"/>
       <c r="R66" s="5" t="inlineStr"/>
       <c r="S66" s="6" t="inlineStr"/>
-      <c r="T66" s="4" t="inlineStr">
-        <is>
-          <t>kode '?' pada: lokasi</t>
-        </is>
-      </c>
+      <c r="T66" s="4" t="inlineStr"/>
     </row>
     <row r="67" ht="110" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -5880,7 +5876,7 @@
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>POHON</t>
         </is>
       </c>
       <c r="K68" s="3" t="inlineStr">
@@ -5916,11 +5912,7 @@
       <c r="Q68" s="5" t="inlineStr"/>
       <c r="R68" s="5" t="inlineStr"/>
       <c r="S68" s="6" t="inlineStr"/>
-      <c r="T68" s="4" t="inlineStr">
-        <is>
-          <t>kode '?' pada: lokasi</t>
-        </is>
-      </c>
+      <c r="T68" s="4" t="inlineStr"/>
     </row>
     <row r="69" ht="110" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -6285,7 +6277,7 @@
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>KLS</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
@@ -6547,7 +6539,7 @@
       </c>
       <c r="M76" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="N76" s="3" t="inlineStr">
@@ -7172,7 +7164,7 @@
       </c>
       <c r="J84" s="3" t="inlineStr">
         <is>
-          <t>POHON</t>
+          <t>TANAH</t>
         </is>
       </c>
       <c r="K84" s="3" t="inlineStr">
@@ -7192,10 +7184,14 @@
       </c>
       <c r="N84" s="3" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O84" s="3" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O84" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/hidayat2024establishing.txt</t>
+        </is>
+      </c>
       <c r="P84" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -7270,10 +7266,14 @@
       </c>
       <c r="N85" s="3" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O85" s="3" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O85" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/hutapea2024palm.txt</t>
+        </is>
+      </c>
       <c r="P85" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -7424,7 +7424,7 @@
       </c>
       <c r="L87" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="M87" s="3" t="inlineStr">
@@ -7750,10 +7750,14 @@
       </c>
       <c r="N91" s="3" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O91" s="3" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O91" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/naftali2024palm.txt</t>
+        </is>
+      </c>
       <c r="P91" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -7910,10 +7914,14 @@
       </c>
       <c r="N93" s="3" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O93" s="3" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O93" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/omar2024outdoor.txt</t>
+        </is>
+      </c>
       <c r="P93" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -8046,7 +8054,7 @@
       </c>
       <c r="J95" s="3" t="inlineStr">
         <is>
-          <t>TANAH</t>
+          <t>POHON</t>
         </is>
       </c>
       <c r="K95" s="3" t="inlineStr">
@@ -8216,7 +8224,7 @@
       </c>
       <c r="L97" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="M97" s="3" t="inlineStr">
@@ -8365,12 +8373,12 @@
       </c>
       <c r="I99" s="3" t="inlineStr">
         <is>
-          <t>KLS</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="J99" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>TANAH</t>
         </is>
       </c>
       <c r="K99" s="3" t="inlineStr">
@@ -8406,11 +8414,7 @@
       <c r="Q99" s="5" t="inlineStr"/>
       <c r="R99" s="5" t="inlineStr"/>
       <c r="S99" s="6" t="inlineStr"/>
-      <c r="T99" s="4" t="inlineStr">
-        <is>
-          <t>kode '?' pada: lokasi</t>
-        </is>
-      </c>
+      <c r="T99" s="4" t="inlineStr"/>
     </row>
     <row r="100" ht="110" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -8466,7 +8470,7 @@
       </c>
       <c r="L100" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="M100" s="3" t="inlineStr">
@@ -8780,7 +8784,7 @@
       </c>
       <c r="J104" s="3" t="inlineStr">
         <is>
-          <t>POHON</t>
+          <t>PABRIK</t>
         </is>
       </c>
       <c r="K104" s="3" t="inlineStr">
@@ -8790,7 +8794,7 @@
       </c>
       <c r="L104" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="M104" s="3" t="inlineStr">
@@ -8853,12 +8857,12 @@
       </c>
       <c r="I105" s="3" t="inlineStr">
         <is>
-          <t>KLS</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="J105" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>POHON</t>
         </is>
       </c>
       <c r="K105" s="3" t="inlineStr">
@@ -8894,11 +8898,7 @@
       <c r="Q105" s="5" t="inlineStr"/>
       <c r="R105" s="5" t="inlineStr"/>
       <c r="S105" s="6" t="inlineStr"/>
-      <c r="T105" s="4" t="inlineStr">
-        <is>
-          <t>kode '?' pada: lokasi</t>
-        </is>
-      </c>
+      <c r="T105" s="4" t="inlineStr"/>
     </row>
     <row r="106" ht="110" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -9513,7 +9513,7 @@
       </c>
       <c r="I113" s="3" t="inlineStr">
         <is>
-          <t>MUTU</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="J113" s="3" t="inlineStr">
@@ -9533,7 +9533,7 @@
       </c>
       <c r="M113" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="N113" s="3" t="inlineStr">
@@ -9600,7 +9600,7 @@
       </c>
       <c r="J114" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>PABRIK</t>
         </is>
       </c>
       <c r="K114" s="3" t="inlineStr">
@@ -9636,11 +9636,7 @@
       <c r="Q114" s="5" t="inlineStr"/>
       <c r="R114" s="5" t="inlineStr"/>
       <c r="S114" s="6" t="inlineStr"/>
-      <c r="T114" s="4" t="inlineStr">
-        <is>
-          <t>kode '?' pada: lokasi</t>
-        </is>
-      </c>
+      <c r="T114" s="4" t="inlineStr"/>
     </row>
     <row r="115" ht="110" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -9862,10 +9858,14 @@
       </c>
       <c r="N117" s="3" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O117" s="3" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O117" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/daud2022loose.txt</t>
+        </is>
+      </c>
       <c r="P117" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -10085,7 +10085,7 @@
       </c>
       <c r="K120" s="3" t="inlineStr">
         <is>
-          <t>RGB+DEPTH</t>
+          <t>RGB</t>
         </is>
       </c>
       <c r="L120" s="3" t="inlineStr">
@@ -10556,7 +10556,7 @@
       </c>
       <c r="J126" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>PABRIK</t>
         </is>
       </c>
       <c r="K126" s="3" t="inlineStr">
@@ -10592,11 +10592,7 @@
       <c r="Q126" s="5" t="inlineStr"/>
       <c r="R126" s="5" t="inlineStr"/>
       <c r="S126" s="6" t="inlineStr"/>
-      <c r="T126" s="4" t="inlineStr">
-        <is>
-          <t>kode '?' pada: lokasi</t>
-        </is>
-      </c>
+      <c r="T126" s="4" t="inlineStr"/>
     </row>
     <row r="127" ht="110" customHeight="1">
       <c r="A127" s="3" t="n">
@@ -10662,10 +10658,14 @@
       </c>
       <c r="N127" s="3" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O127" s="3" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O127" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/aji2021automatic.txt</t>
+        </is>
+      </c>
       <c r="P127" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -10899,7 +10899,7 @@
       </c>
       <c r="M130" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="N130" s="3" t="inlineStr">
@@ -11210,12 +11210,12 @@
       </c>
       <c r="L134" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="M134" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="N134" s="3" t="inlineStr">
@@ -11287,7 +11287,7 @@
       </c>
       <c r="K135" s="3" t="inlineStr">
         <is>
-          <t>MSI+TERMAL</t>
+          <t>RGB+TERMAL</t>
         </is>
       </c>
       <c r="L135" s="3" t="inlineStr">
@@ -11297,7 +11297,7 @@
       </c>
       <c r="M135" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="N135" s="3" t="inlineStr">
@@ -11675,7 +11675,7 @@
       </c>
       <c r="I140" s="3" t="inlineStr">
         <is>
-          <t>SENSOR</t>
+          <t>MUTU</t>
         </is>
       </c>
       <c r="J140" s="3" t="inlineStr">
@@ -11685,17 +11685,17 @@
       </c>
       <c r="K140" s="3" t="inlineStr">
         <is>
-          <t>MSI</t>
+          <t>RGB</t>
         </is>
       </c>
       <c r="L140" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="M140" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="N140" s="3" t="inlineStr">
@@ -11762,7 +11762,7 @@
       </c>
       <c r="J141" s="3" t="inlineStr">
         <is>
-          <t>PABRIK</t>
+          <t>TANAH</t>
         </is>
       </c>
       <c r="K141" s="3" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="I144" s="3" t="inlineStr">
         <is>
-          <t>KLS</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="J144" s="3" t="inlineStr">
@@ -12019,7 +12019,7 @@
       </c>
       <c r="M144" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="N144" s="3" t="inlineStr">
@@ -12860,14 +12860,14 @@
     </row>
     <row r="155" ht="110" customHeight="1">
       <c r="A155" s="3" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B155" s="3" t="n">
-        <v>2175</v>
+        <v>2190</v>
       </c>
       <c r="C155" s="3" t="inlineStr">
         <is>
-          <t>jupriyanto2018uav</t>
+          <t>sabri2018evaluation</t>
         </is>
       </c>
       <c r="D155" s="3" t="inlineStr">
@@ -12877,17 +12877,17 @@
       </c>
       <c r="E155" s="4" t="inlineStr">
         <is>
-          <t>UAV application for oil palm harvest prediction</t>
+          <t>Evaluation of color models for palm oil fresh fruit bunch ripeness classification</t>
         </is>
       </c>
       <c r="F155" s="3" t="inlineStr">
         <is>
-          <t>10.1088/1742-6596/1130/1/012001</t>
+          <t>10.11591/ijeecs.v11.i2.pp549-557</t>
         </is>
       </c>
       <c r="G155" s="4" t="inlineStr">
         <is>
-          <t>Determination of UAV system configuration for oil palm harvest prediction application is an important step in plantation production maximization. The objective of this paper is to demonstrate how UAV systems can be used to produce high-resolution images that can be used to predict crops. The study is divided into two stages: UAV system configuration analysis and digital image processing to predict the crop. The UAV system configuration analysis consists of airframe, propulsion, avionic and ground control station. Airborne systems use a X-8 airframe controlled with Pixhawk avionics, electric motors, and a 20.2 Mega Pixel digital camera. The UAV system is used to produce a high-resolution digital image on a 6-year-old oil palm plantation in Labuhan Batu Utara, North Sumatra. This UAV system produces high-resolution digital image that can be used to calculate the number of plants. The number of plants in this particular area is then used as input to predict the crop. Estimated harvests of 6-year-old oil palm plantations produce an average of 50.5 tons per year per hectare. This result is bigger than the one of palm oil plantation management’s estimation company which is 23 tons per year per ha.</t>
+          <t>This paper investigates the application of eight color models for automatic palm oil Fresh Fruit Bunch (FFB) ripeness classification with multi-class Support Vector Machine (SVM).  Ripeness classification is important during harvesting to ensure that they are harvested during the correct ripe stage for optimum oil production.  Since color is a significant indicator for agriculturists to determine the ripeness of FFB, it is critical to determine the right color model. Eight color models have been investigated namely, HSV, I1I2I3, LAB, XYZ, YCbCr, YIQ, YUV and RGB. Color moments were extracted from each of these color models for the classification of four stages of FFB ripeness that are unripe, under-ripe, ripe and over-ripe.  A database of five hundred images of palm oil FFB has been constructed and experiments showed that YCbCr and YUV outperform the other color models.</t>
         </is>
       </c>
       <c r="H155" s="3" t="inlineStr">
@@ -12897,12 +12897,12 @@
       </c>
       <c r="I155" s="3" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>KLS</t>
         </is>
       </c>
       <c r="J155" s="3" t="inlineStr">
         <is>
-          <t>UAV</t>
+          <t>?</t>
         </is>
       </c>
       <c r="K155" s="3" t="inlineStr">
@@ -12917,7 +12917,7 @@
       </c>
       <c r="M155" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="N155" s="3" t="inlineStr">
@@ -12927,7 +12927,7 @@
       </c>
       <c r="O155" s="3" t="inlineStr">
         <is>
-          <t>literature/scopus-2026-09/teks/jupriyanto2018uav.txt</t>
+          <t>literature/scopus-2026-09/teks/sabri2018evaluation.txt</t>
         </is>
       </c>
       <c r="P155" s="3" t="inlineStr">
@@ -12938,18 +12938,22 @@
       <c r="Q155" s="5" t="inlineStr"/>
       <c r="R155" s="5" t="inlineStr"/>
       <c r="S155" s="6" t="inlineStr"/>
-      <c r="T155" s="4" t="inlineStr"/>
+      <c r="T155" s="4" t="inlineStr">
+        <is>
+          <t>kode '?' pada: lokasi</t>
+        </is>
+      </c>
     </row>
     <row r="156" ht="110" customHeight="1">
       <c r="A156" s="3" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B156" s="3" t="n">
-        <v>2190</v>
+        <v>2209</v>
       </c>
       <c r="C156" s="3" t="inlineStr">
         <is>
-          <t>sabri2018evaluation</t>
+          <t>salambue2018investigation</t>
         </is>
       </c>
       <c r="D156" s="3" t="inlineStr">
@@ -12959,17 +12963,17 @@
       </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
-          <t>Evaluation of color models for palm oil fresh fruit bunch ripeness classification</t>
+          <t>Investigation of the ripeness of oil palm fresh fruit bunches using bio-speckle imaging</t>
         </is>
       </c>
       <c r="F156" s="3" t="inlineStr">
         <is>
-          <t>10.11591/ijeecs.v11.i2.pp549-557</t>
+          <t>10.1088/1742-6596/978/1/012071</t>
         </is>
       </c>
       <c r="G156" s="4" t="inlineStr">
         <is>
-          <t>This paper investigates the application of eight color models for automatic palm oil Fresh Fruit Bunch (FFB) ripeness classification with multi-class Support Vector Machine (SVM).  Ripeness classification is important during harvesting to ensure that they are harvested during the correct ripe stage for optimum oil production.  Since color is a significant indicator for agriculturists to determine the ripeness of FFB, it is critical to determine the right color model. Eight color models have been investigated namely, HSV, I1I2I3, LAB, XYZ, YCbCr, YIQ, YUV and RGB. Color moments were extracted from each of these color models for the classification of four stages of FFB ripeness that are unripe, under-ripe, ripe and over-ripe.  A database of five hundred images of palm oil FFB has been constructed and experiments showed that YCbCr and YUV outperform the other color models.</t>
+          <t>The ripeness of the oil palm Fresh Fruit Bunches (FFB) determines the yield of the oil produced. Traditionally there are two ways to determine FFB ripeness which are the number of loose fruits and the color changes. Nevertheless, one drawback of visual determination is subjective and qualitative judgment. In this study, the FFB ripeness was investigated using laser based image processing technique. The advantages of using this technique are non-destructive, simple and quantitative. The working principle of the investigation is that a FFB is inserted into a light tight box which contains a laser diode and a CMOS camera, the FFB is illuminated, and then an image is recorded. The FFB image recorder was performed on four FFB fractions i.e. F0, F3, F4 and F5 on the front and rear surfaces at three sections. The recorded images are speckled granules that have light intensity variation (bio-speckle imaging). The feature extracted from the specked image is the contrast value obtained from the average gray value intensity and the standard deviation. Based on the contrast values, the four fractions of FFB can be grouped into three levels of ripeness of unripe (F0), ripe (F3) and overripe (F4 and F5) on the front surface of base section of FFB by 75%.</t>
         </is>
       </c>
       <c r="H156" s="3" t="inlineStr">
@@ -12979,17 +12983,17 @@
       </c>
       <c r="I156" s="3" t="inlineStr">
         <is>
-          <t>KLS</t>
+          <t>SENSOR</t>
         </is>
       </c>
       <c r="J156" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>PABRIK</t>
         </is>
       </c>
       <c r="K156" s="3" t="inlineStr">
         <is>
-          <t>RGB</t>
+          <t>LASER</t>
         </is>
       </c>
       <c r="L156" s="3" t="inlineStr">
@@ -13009,7 +13013,7 @@
       </c>
       <c r="O156" s="3" t="inlineStr">
         <is>
-          <t>literature/scopus-2026-09/teks/sabri2018evaluation.txt</t>
+          <t>literature/scopus-2026-09/teks/salambue2018investigation.txt</t>
         </is>
       </c>
       <c r="P156" s="3" t="inlineStr">
@@ -13020,22 +13024,18 @@
       <c r="Q156" s="5" t="inlineStr"/>
       <c r="R156" s="5" t="inlineStr"/>
       <c r="S156" s="6" t="inlineStr"/>
-      <c r="T156" s="4" t="inlineStr">
-        <is>
-          <t>kode '?' pada: lokasi</t>
-        </is>
-      </c>
+      <c r="T156" s="4" t="inlineStr"/>
     </row>
     <row r="157" ht="110" customHeight="1">
       <c r="A157" s="3" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B157" s="3" t="n">
-        <v>2209</v>
+        <v>2203</v>
       </c>
       <c r="C157" s="3" t="inlineStr">
         <is>
-          <t>salambue2018investigation</t>
+          <t>siddesha2018segmentation</t>
         </is>
       </c>
       <c r="D157" s="3" t="inlineStr">
@@ -13045,17 +13045,17 @@
       </c>
       <c r="E157" s="4" t="inlineStr">
         <is>
-          <t>Investigation of the ripeness of oil palm fresh fruit bunches using bio-speckle imaging</t>
+          <t>Segmentation of oil palm crop bunch from tree images</t>
         </is>
       </c>
       <c r="F157" s="3" t="inlineStr">
         <is>
-          <t>10.1088/1742-6596/978/1/012071</t>
+          <t>10.1109/smarttechcon.2017.8358639</t>
         </is>
       </c>
       <c r="G157" s="4" t="inlineStr">
         <is>
-          <t>The ripeness of the oil palm Fresh Fruit Bunches (FFB) determines the yield of the oil produced. Traditionally there are two ways to determine FFB ripeness which are the number of loose fruits and the color changes. Nevertheless, one drawback of visual determination is subjective and qualitative judgment. In this study, the FFB ripeness was investigated using laser based image processing technique. The advantages of using this technique are non-destructive, simple and quantitative. The working principle of the investigation is that a FFB is inserted into a light tight box which contains a laser diode and a CMOS camera, the FFB is illuminated, and then an image is recorded. The FFB image recorder was performed on four FFB fractions i.e. F0, F3, F4 and F5 on the front and rear surfaces at three sections. The recorded images are speckled granules that have light intensity variation (bio-speckle imaging). The feature extracted from the specked image is the contrast value obtained from the average gray value intensity and the standard deviation. Based on the contrast values, the four fractions of FFB can be grouped into three levels of ripeness of unripe (F0), ripe (F3) and overripe (F4 and F5) on the front surface of base section of FFB by 75%.</t>
+          <t>Segmentation is one of the challenging step in image analysis. It is very cumbersome process for the region with complex background. Segmentation techniques can be either of supervised or unsupervised in nature. In this paper, we explored both supervised and unsupervised techniques for the segmentation of oil palm crop bunch from the tree image. This work has a vital importance in Harvesting which is one of the important stages in crop management. Right time and proper crop harvesting will enhance the quality. Here we explored Hill climbing, Growcut, Random Walker and MSRM algorithm as a part of supervised techniques and K-Means, Fuzzy-C-Means as un-supervised techniques. The performance of these algorithms are demonstrated by conducting experiment with dataset of 100 images.</t>
         </is>
       </c>
       <c r="H157" s="3" t="inlineStr">
@@ -13065,17 +13065,17 @@
       </c>
       <c r="I157" s="3" t="inlineStr">
         <is>
-          <t>SENSOR</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="J157" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>POHON</t>
         </is>
       </c>
       <c r="K157" s="3" t="inlineStr">
         <is>
-          <t>LASER</t>
+          <t>RGB</t>
         </is>
       </c>
       <c r="L157" s="3" t="inlineStr">
@@ -13085,19 +13085,15 @@
       </c>
       <c r="M157" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="N157" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="O157" s="3" t="inlineStr">
-        <is>
-          <t>literature/scopus-2026-09/teks/salambue2018investigation.txt</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O157" s="3" t="inlineStr"/>
       <c r="P157" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -13106,42 +13102,38 @@
       <c r="Q157" s="5" t="inlineStr"/>
       <c r="R157" s="5" t="inlineStr"/>
       <c r="S157" s="6" t="inlineStr"/>
-      <c r="T157" s="4" t="inlineStr">
-        <is>
-          <t>kode '?' pada: lokasi</t>
-        </is>
-      </c>
+      <c r="T157" s="4" t="inlineStr"/>
     </row>
     <row r="158" ht="110" customHeight="1">
       <c r="A158" s="3" t="n">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B158" s="3" t="n">
-        <v>2203</v>
+        <v>2237</v>
       </c>
       <c r="C158" s="3" t="inlineStr">
         <is>
-          <t>siddesha2018segmentation</t>
+          <t>pamornnak2017automatic</t>
         </is>
       </c>
       <c r="D158" s="3" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2017</t>
         </is>
       </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
-          <t>Segmentation of oil palm crop bunch from tree images</t>
+          <t>An automatic and rapid system for grading palm bunch using a Kinect camera</t>
         </is>
       </c>
       <c r="F158" s="3" t="inlineStr">
         <is>
-          <t>10.1109/smarttechcon.2017.8358639</t>
+          <t>10.1016/j.compag.2017.10.020</t>
         </is>
       </c>
       <c r="G158" s="4" t="inlineStr">
         <is>
-          <t>Segmentation is one of the challenging step in image analysis. It is very cumbersome process for the region with complex background. Segmentation techniques can be either of supervised or unsupervised in nature. In this paper, we explored both supervised and unsupervised techniques for the segmentation of oil palm crop bunch from the tree image. This work has a vital importance in Harvesting which is one of the important stages in crop management. Right time and proper crop harvesting will enhance the quality. Here we explored Hill climbing, Growcut, Random Walker and MSRM algorithm as a part of supervised techniques and K-Means, Fuzzy-C-Means as un-supervised techniques. The performance of these algorithms are demonstrated by conducting experiment with dataset of 100 images.</t>
+          <t>In a trading market, price of oil palm (Elaeis guineensis) is negotiated depending some key parameters of the fresh fruit bunch (FFB). Inspectors have been hired by a buyer to grade FFB to accept or reject. The classification results made by human inspection are skeptical and not very reliable if workload is high. We have developed a system to grade FFB depending on its quality. Several palm features are extracted from RGB, near infrared, and depth images, captured with a Microsoft Kinect camera version 2.0 installed in a light-controlled environment on the conveyor line. Two main algorithms for classification have been developed. The first algorithm is called a volume integration scheme (SVIS), which measures the relative volume of palm bunch. The second developed algorithm classifies palm bunch into three grades (L-Grade, M-Grade and H-Grade) based on oil content from Soxhlet extraction. The system achieves 83% accuracy for grading palm bunch within 6 s per one sample, which shows the possibility of using the system in a trading market.</t>
         </is>
       </c>
       <c r="H158" s="3" t="inlineStr">
@@ -13151,17 +13143,17 @@
       </c>
       <c r="I158" s="3" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>MUTU</t>
         </is>
       </c>
       <c r="J158" s="3" t="inlineStr">
         <is>
-          <t>POHON</t>
+          <t>PABRIK</t>
         </is>
       </c>
       <c r="K158" s="3" t="inlineStr">
         <is>
-          <t>RGB</t>
+          <t>RGB+NIR+DEPTH</t>
         </is>
       </c>
       <c r="L158" s="3" t="inlineStr">
@@ -13171,7 +13163,7 @@
       </c>
       <c r="M158" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="N158" s="3" t="inlineStr">
@@ -13192,14 +13184,14 @@
     </row>
     <row r="159" ht="110" customHeight="1">
       <c r="A159" s="3" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B159" s="3" t="n">
-        <v>2237</v>
+        <v>2282</v>
       </c>
       <c r="C159" s="3" t="inlineStr">
         <is>
-          <t>pamornnak2017automatic</t>
+          <t>shiddiq2017ripeness</t>
         </is>
       </c>
       <c r="D159" s="3" t="inlineStr">
@@ -13209,17 +13201,17 @@
       </c>
       <c r="E159" s="4" t="inlineStr">
         <is>
-          <t>An automatic and rapid system for grading palm bunch using a Kinect camera</t>
+          <t>Ripeness detection simulation of oil palm fruit bunches using laser-based imaging system</t>
         </is>
       </c>
       <c r="F159" s="3" t="inlineStr">
         <is>
-          <t>10.1016/j.compag.2017.10.020</t>
+          <t>10.1063/1.4973101</t>
         </is>
       </c>
       <c r="G159" s="4" t="inlineStr">
         <is>
-          <t>In a trading market, price of oil palm (Elaeis guineensis) is negotiated depending some key parameters of the fresh fruit bunch (FFB). Inspectors have been hired by a buyer to grade FFB to accept or reject. The classification results made by human inspection are skeptical and not very reliable if workload is high. We have developed a system to grade FFB depending on its quality. Several palm features are extracted from RGB, near infrared, and depth images, captured with a Microsoft Kinect camera version 2.0 installed in a light-controlled environment on the conveyor line. Two main algorithms for classification have been developed. The first algorithm is called a volume integration scheme (SVIS), which measures the relative volume of palm bunch. The second developed algorithm classifies palm bunch into three grades (L-Grade, M-Grade and H-Grade) based on oil content from Soxhlet extraction. The system achieves 83% accuracy for grading palm bunch within 6 s per one sample, which shows the possibility of using the system in a trading market.</t>
+          <t>Ripeness is one of important factors for quality sorting of harvested oil palm fresh fruit bunches (FFB). Traditional ripeness classifications using FFB color and number of fruit loose for harvesting have some disadvantages especially for high oil palm trees. A laser based imaging system is proposed to substitute the traditional method. In this study, ripeness detection simulation of oil palm FFBs was performed. The system composed of two diode lasers with 532 nm and 680 nm in wavelengths and a CMOS camera which was set on a rotating plate for easy adjustment of laser beam hitting FFB. The FFB samples were placed on an aluminum platform with 4 height variations, 1.5 m, 2 m, 2.5 m, and 3 m. The relations of reflectance intensities represented by Red Green Blue (RGB) values of the FFB images to the height variations and ripeness levels of FFBs with and without laser beam were analyzed. The samples were from Tenera variety with 4 ripeness levels called F0, F1, F3, and F4. The results showed that the red component of RGB values were dominant for FFBs without laser and with red laser. The average RGB values are higher for F3 (ripe) level and F4 (overripe). Imaging with green laser showed consistency. Imaging methods using laser was able to differentiate ripeness levels of oil palm fresh fruit bunch, it could be applied for future remote detection of oil palm FFB ripeness.</t>
         </is>
       </c>
       <c r="H159" s="3" t="inlineStr">
@@ -13229,7 +13221,7 @@
       </c>
       <c r="I159" s="3" t="inlineStr">
         <is>
-          <t>KLS</t>
+          <t>SENSOR</t>
         </is>
       </c>
       <c r="J159" s="3" t="inlineStr">
@@ -13239,7 +13231,7 @@
       </c>
       <c r="K159" s="3" t="inlineStr">
         <is>
-          <t>RGB+NIR+DEPTH</t>
+          <t>RGB+LASER</t>
         </is>
       </c>
       <c r="L159" s="3" t="inlineStr">
@@ -13270,34 +13262,34 @@
     </row>
     <row r="160" ht="110" customHeight="1">
       <c r="A160" s="3" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B160" s="3" t="n">
-        <v>2282</v>
+        <v>2311</v>
       </c>
       <c r="C160" s="3" t="inlineStr">
         <is>
-          <t>shiddiq2017ripeness</t>
+          <t>shabdin2016study</t>
         </is>
       </c>
       <c r="D160" s="3" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2016</t>
         </is>
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
-          <t>Ripeness detection simulation of oil palm fruit bunches using laser-based imaging system</t>
+          <t>A study on the oil palm fresh fruit bunch (FFB) ripeness detection by using Hue, Saturation and Intensity (HSI) approach</t>
         </is>
       </c>
       <c r="F160" s="3" t="inlineStr">
         <is>
-          <t>10.1063/1.4973101</t>
+          <t>10.1088/1755-1315/37/1/012039</t>
         </is>
       </c>
       <c r="G160" s="4" t="inlineStr">
         <is>
-          <t>Ripeness is one of important factors for quality sorting of harvested oil palm fresh fruit bunches (FFB). Traditional ripeness classifications using FFB color and number of fruit loose for harvesting have some disadvantages especially for high oil palm trees. A laser based imaging system is proposed to substitute the traditional method. In this study, ripeness detection simulation of oil palm FFBs was performed. The system composed of two diode lasers with 532 nm and 680 nm in wavelengths and a CMOS camera which was set on a rotating plate for easy adjustment of laser beam hitting FFB. The FFB samples were placed on an aluminum platform with 4 height variations, 1.5 m, 2 m, 2.5 m, and 3 m. The relations of reflectance intensities represented by Red Green Blue (RGB) values of the FFB images to the height variations and ripeness levels of FFBs with and without laser beam were analyzed. The samples were from Tenera variety with 4 ripeness levels called F0, F1, F3, and F4. The results showed that the red component of RGB values were dominant for FFBs without laser and with red laser. The average RGB values are higher for F3 (ripe) level and F4 (overripe). Imaging with green laser showed consistency. Imaging methods using laser was able to differentiate ripeness levels of oil palm fresh fruit bunch, it could be applied for future remote detection of oil palm FFB ripeness.</t>
+          <t>To increase the quality of palm oil means to accurately grade the oil palm fresh fruit bunches (FFB) for processing. In this paper, HSI color model was used to determine the relationship between FFB ’ s color with the underipe and ripe category so that the grading system could be accurately done. From the analysis manipulation, a formula was generated and applied to the data obtained. The by linear regression in the data shows an average success rate at 45% accuracy for oil palm ripeness detection. Artificial Neural Network (ANN) however return a better accuracy result for both underipe and ripe categories which are 60% and 80% respectively. This yield an overall accuracy of 70%. This can be increased more by improving the grading system.</t>
         </is>
       </c>
       <c r="H160" s="3" t="inlineStr">
@@ -13307,17 +13299,17 @@
       </c>
       <c r="I160" s="3" t="inlineStr">
         <is>
-          <t>SENSOR</t>
+          <t>KLS</t>
         </is>
       </c>
       <c r="J160" s="3" t="inlineStr">
         <is>
-          <t>POHON</t>
+          <t>PABRIK</t>
         </is>
       </c>
       <c r="K160" s="3" t="inlineStr">
         <is>
-          <t>RGB+LASER</t>
+          <t>RGB</t>
         </is>
       </c>
       <c r="L160" s="3" t="inlineStr">
@@ -13332,10 +13324,14 @@
       </c>
       <c r="N160" s="3" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O160" s="3" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O160" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/shabdin2016study.txt</t>
+        </is>
+      </c>
       <c r="P160" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -13348,34 +13344,34 @@
     </row>
     <row r="161" ht="110" customHeight="1">
       <c r="A161" s="3" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B161" s="3" t="n">
-        <v>2311</v>
+        <v>2369</v>
       </c>
       <c r="C161" s="3" t="inlineStr">
         <is>
-          <t>shabdin2016study</t>
+          <t>cherie2015advance</t>
         </is>
       </c>
       <c r="D161" s="3" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2015</t>
         </is>
       </c>
       <c r="E161" s="4" t="inlineStr">
         <is>
-          <t>A study on the oil palm fresh fruit bunch (FFB) ripeness detection by using Hue, Saturation and Intensity (HSI) approach</t>
+          <t>Advance models for camera-vision based oil content prediction of intact oil palm fruits (Elaeis Guineensis Jacq) on trees with nondestructive evaluation</t>
         </is>
       </c>
       <c r="F161" s="3" t="inlineStr">
         <is>
-          <t>10.1088/1755-1315/37/1/012039</t>
+          <t>10.18517/ijaseit.5.4.542</t>
         </is>
       </c>
       <c r="G161" s="4" t="inlineStr">
         <is>
-          <t>To increase the quality of palm oil means to accurately grade the oil palm fresh fruit bunches (FFB) for processing. In this paper, HSI color model was used to determine the relationship between FFB ’ s color with the underipe and ripe category so that the grading system could be accurately done. From the analysis manipulation, a formula was generated and applied to the data obtained. The by linear regression in the data shows an average success rate at 45% accuracy for oil palm ripeness detection. Artificial Neural Network (ANN) however return a better accuracy result for both underipe and ripe categories which are 60% and 80% respectively. This yield an overall accuracy of 70%. This can be increased more by improving the grading system.</t>
+          <t>In this study, the correlation between oil palm fresh fruits bunch (FFB) appearance and its oil content (OC) was explored. FFB samples were recorded from various distance (2, 7, and 10 m) with different lighting spectrums and configurations (Ultraviolet: 280-380nm, Visible: 400-700nm, and Infrared: 720-1100nm) and intensities (600watt and 1000watt lamps) to explore the correlations. The recorded FFB images were segmented and its color features were subsequently extracted to be used as input variables for modeling the OC of the FFB. In this study, four developed models were selected to perform oil content prediction (OCP) for intact FFBs. These models were selected based on their validity and accuracy upon performing the OCP. Models were developed using Multi-Linear-Perceptron-Artificial-Neural-Network (MLP-ANN) methods, employing 10 hidden layers and 15 images features as input variables. Statistical engineering software was used to create the models. Although the number of FFB samples in this study was limited, four models were successfully developed to predict intact FFB’s OC, based on its images’ color features. Three OCP models developed for image recording from 10 m under UV, Vis2, and IR2 lighting configurations. Another model was successfully developed for short range imaging (2m) under IR2 light. The coefficient of correlation for each model when validated was 0.816, 0.902, 0.919, and 0.886, respectively. For bias and error, these selected models obtained root-mean-square error (RMSE) of 1.803, 0.753, 0.607, and 1.104, respectively.</t>
         </is>
       </c>
       <c r="H161" s="3" t="inlineStr">
@@ -13385,17 +13381,17 @@
       </c>
       <c r="I161" s="3" t="inlineStr">
         <is>
-          <t>KLS</t>
+          <t>MUTU</t>
         </is>
       </c>
       <c r="J161" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>POHON</t>
         </is>
       </c>
       <c r="K161" s="3" t="inlineStr">
         <is>
-          <t>RGB</t>
+          <t>RGB+NIR</t>
         </is>
       </c>
       <c r="L161" s="3" t="inlineStr">
@@ -13405,19 +13401,15 @@
       </c>
       <c r="M161" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="N161" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="O161" s="3" t="inlineStr">
-        <is>
-          <t>literature/scopus-2026-09/teks/shabdin2016study.txt</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O161" s="3" t="inlineStr"/>
       <c r="P161" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -13426,22 +13418,18 @@
       <c r="Q161" s="5" t="inlineStr"/>
       <c r="R161" s="5" t="inlineStr"/>
       <c r="S161" s="6" t="inlineStr"/>
-      <c r="T161" s="4" t="inlineStr">
-        <is>
-          <t>kode '?' pada: lokasi</t>
-        </is>
-      </c>
+      <c r="T161" s="4" t="inlineStr"/>
     </row>
     <row r="162" ht="110" customHeight="1">
       <c r="A162" s="3" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B162" s="3" t="n">
-        <v>2369</v>
+        <v>2358</v>
       </c>
       <c r="C162" s="3" t="inlineStr">
         <is>
-          <t>cherie2015advance</t>
+          <t>pamornnak2015oil</t>
         </is>
       </c>
       <c r="D162" s="3" t="inlineStr">
@@ -13451,17 +13439,17 @@
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
-          <t>Advance models for camera-vision based oil content prediction of intact oil palm fruits (Elaeis Guineensis Jacq) on trees with nondestructive evaluation</t>
+          <t>Oil content determination scheme of postharvest oil palm for mobile devices</t>
         </is>
       </c>
       <c r="F162" s="3" t="inlineStr">
         <is>
-          <t>10.18517/ijaseit.5.4.542</t>
+          <t>10.1016/j.biosystemseng.2015.03.010</t>
         </is>
       </c>
       <c r="G162" s="4" t="inlineStr">
         <is>
-          <t>In this study, the correlation between oil palm fresh fruits bunch (FFB) appearance and its oil content (OC) was explored. FFB samples were recorded from various distance (2, 7, and 10 m) with different lighting spectrums and configurations (Ultraviolet: 280-380nm, Visible: 400-700nm, and Infrared: 720-1100nm) and intensities (600watt and 1000watt lamps) to explore the correlations. The recorded FFB images were segmented and its color features were subsequently extracted to be used as input variables for modeling the OC of the FFB. In this study, four developed models were selected to perform oil content prediction (OCP) for intact FFBs. These models were selected based on their validity and accuracy upon performing the OCP. Models were developed using Multi-Linear-Perceptron-Artificial-Neural-Network (MLP-ANN) methods, employing 10 hidden layers and 15 images features as input variables. Statistical engineering software was used to create the models. Although the number of FFB samples in this study was limited, four models were successfully developed to predict intact FFB’s OC, based on its images’ color features. Three OCP models developed for image recording from 10 m under UV, Vis2, and IR2 lighting configurations. Another model was successfully developed for short range imaging (2m) under IR2 light. The coefficient of correlation for each model when validated was 0.816, 0.902, 0.919, and 0.886, respectively. For bias and error, these selected models obtained root-mean-square error (RMSE) of 1.803, 0.753, 0.607, and 1.104, respectively.</t>
+          <t>In this paper, a simple scheme based on an image processing technique for determining oil content in postharvest oil palm (Elaeis guineensis Jacq.), implemented for a mobile device, is proposed. The scheme has three main algorithms for colour correction, classification and oil extraction rate (OER) determination. The colour correction algorithm can correct image colour from the device-dependence effect in the standard RGB (sRGB) colour model based on the determined device profile function. The classification process was developed on a two-layer feedforward neural network by using features from the hue value of oil palm fruits. The OER determination function was modelled by using a polynomial regression model based on the hue and saturation values. The results demonstrated that the proposed scheme can classify and determine the OER with a simple calculation. The scheme was implemented on a mobile device/phone and tested with 64 oil palm fruit samples. Compared with the standard Soxhlet extraction measurement, the scheme achieves a mean error of OER 2.20 with a postharvest OER range of 30–73%.</t>
         </is>
       </c>
       <c r="H162" s="3" t="inlineStr">
@@ -13476,7 +13464,7 @@
       </c>
       <c r="J162" s="3" t="inlineStr">
         <is>
-          <t>POHON</t>
+          <t>PABRIK</t>
         </is>
       </c>
       <c r="K162" s="3" t="inlineStr">
@@ -13491,7 +13479,7 @@
       </c>
       <c r="M162" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="N162" s="3" t="inlineStr">
@@ -13512,14 +13500,14 @@
     </row>
     <row r="163" ht="110" customHeight="1">
       <c r="A163" s="3" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B163" s="3" t="n">
-        <v>2358</v>
+        <v>2348</v>
       </c>
       <c r="C163" s="3" t="inlineStr">
         <is>
-          <t>pamornnak2015oil</t>
+          <t>taparugssanagorn2015non</t>
         </is>
       </c>
       <c r="D163" s="3" t="inlineStr">
@@ -13529,17 +13517,17 @@
       </c>
       <c r="E163" s="4" t="inlineStr">
         <is>
-          <t>Oil content determination scheme of postharvest oil palm for mobile devices</t>
+          <t>A non-destructive oil palm ripeness recognition system using relative entropy</t>
         </is>
       </c>
       <c r="F163" s="3" t="inlineStr">
         <is>
-          <t>10.1016/j.biosystemseng.2015.03.010</t>
+          <t>10.1016/j.compag.2015.09.018</t>
         </is>
       </c>
       <c r="G163" s="4" t="inlineStr">
         <is>
-          <t>In this paper, a simple scheme based on an image processing technique for determining oil content in postharvest oil palm (Elaeis guineensis Jacq.), implemented for a mobile device, is proposed. The scheme has three main algorithms for colour correction, classification and oil extraction rate (OER) determination. The colour correction algorithm can correct image colour from the device-dependence effect in the standard RGB (sRGB) colour model based on the determined device profile function. The classification process was developed on a two-layer feedforward neural network by using features from the hue value of oil palm fruits. The OER determination function was modelled by using a polynomial regression model based on the hue and saturation values. The results demonstrated that the proposed scheme can classify and determine the OER with a simple calculation. The scheme was implemented on a mobile device/phone and tested with 64 oil palm fruit samples. Compared with the standard Soxhlet extraction measurement, the scheme achieves a mean error of OER 2.20 with a postharvest OER range of 30–73%.</t>
+          <t>This paper introduces a relative entropy based image processing approach for the non-destructive prediction of the maturity of oil palm fresh fruit bunches (FFB) which enables the determination of the correct time for harvesting. The results of an experimental study of applying the Kullback–Leibler distance to the problem of oil palm classification are presented. It is shown that the proposed algorithm has an excellent accuracy and it can be computed very fast. The overall proposed system is simple and useful for oil palm farmers and entrepreneurs.</t>
         </is>
       </c>
       <c r="H163" s="3" t="inlineStr">
@@ -13549,12 +13537,12 @@
       </c>
       <c r="I163" s="3" t="inlineStr">
         <is>
-          <t>MUTU</t>
+          <t>KLS</t>
         </is>
       </c>
       <c r="J163" s="3" t="inlineStr">
         <is>
-          <t>PABRIK</t>
+          <t>?</t>
         </is>
       </c>
       <c r="K163" s="3" t="inlineStr">
@@ -13569,7 +13557,7 @@
       </c>
       <c r="M163" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="N163" s="3" t="inlineStr">
@@ -13586,38 +13574,42 @@
       <c r="Q163" s="5" t="inlineStr"/>
       <c r="R163" s="5" t="inlineStr"/>
       <c r="S163" s="6" t="inlineStr"/>
-      <c r="T163" s="4" t="inlineStr"/>
+      <c r="T163" s="4" t="inlineStr">
+        <is>
+          <t>kode '?' pada: lokasi</t>
+        </is>
+      </c>
     </row>
     <row r="164" ht="110" customHeight="1">
       <c r="A164" s="3" t="n">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B164" s="3" t="n">
-        <v>2348</v>
+        <v>2405</v>
       </c>
       <c r="C164" s="3" t="inlineStr">
         <is>
-          <t>taparugssanagorn2015non</t>
+          <t>alfatni2014oilb</t>
         </is>
       </c>
       <c r="D164" s="3" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>A non-destructive oil palm ripeness recognition system using relative entropy</t>
+          <t>Oil palm fresh fruit bunch ripeness classification based on rule-based expert system of ROI image processing technique results</t>
         </is>
       </c>
       <c r="F164" s="3" t="inlineStr">
         <is>
-          <t>10.1016/j.compag.2015.09.018</t>
+          <t>10.1088/1755-1315/20/1/012018</t>
         </is>
       </c>
       <c r="G164" s="4" t="inlineStr">
         <is>
-          <t>This paper introduces a relative entropy based image processing approach for the non-destructive prediction of the maturity of oil palm fresh fruit bunches (FFB) which enables the determination of the correct time for harvesting. The results of an experimental study of applying the Kullback–Leibler distance to the problem of oil palm classification are presented. It is shown that the proposed algorithm has an excellent accuracy and it can be computed very fast. The overall proposed system is simple and useful for oil palm farmers and entrepreneurs.</t>
+          <t>There is a processing need for a fast, easy and accurate classification system for oil palm fruit ripeness. Such a system will be invaluable to farmers and plantation managers who need to sell their oil palm fresh fruit bunch (FFB) for the mill as this will avoid disputes. In this paper,a new approach was developed under the name of expert rules-based systembased on the image processing techniques results of thethree different oil palm FFB region of interests (ROIs), namely; ROI1 (300x300 pixels), ROI2 (50x50 pixels) and ROI3 (100x100 pixels). The results show that the best rule-based ROIs for statistical colour feature extraction with k-nearest neighbors (KNN) classifier at 94% were chosen as well as the ROIs that indicated results higher than the rule-based outcome, such as the ROIs of statistical colour feature extraction with artificial neural network (ANN) classifier at 94%, were selected for further FFB ripeness inspection system.</t>
         </is>
       </c>
       <c r="H164" s="3" t="inlineStr">
@@ -13672,14 +13664,14 @@
     </row>
     <row r="165" ht="110" customHeight="1">
       <c r="A165" s="3" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B165" s="3" t="n">
-        <v>2405</v>
+        <v>2409</v>
       </c>
       <c r="C165" s="3" t="inlineStr">
         <is>
-          <t>alfatni2014oilb</t>
+          <t>bensaeed2014oil</t>
         </is>
       </c>
       <c r="D165" s="3" t="inlineStr">
@@ -13689,17 +13681,17 @@
       </c>
       <c r="E165" s="4" t="inlineStr">
         <is>
-          <t>Oil palm fresh fruit bunch ripeness classification based on rule-based expert system of ROI image processing technique results</t>
+          <t>Oil palm fruit grading using a hyperspectral device and machine learning algorithm</t>
         </is>
       </c>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>10.1088/1755-1315/20/1/012018</t>
+          <t>10.1088/1755-1315/20/1/012017</t>
         </is>
       </c>
       <c r="G165" s="4" t="inlineStr">
         <is>
-          <t>There is a processing need for a fast, easy and accurate classification system for oil palm fruit ripeness. Such a system will be invaluable to farmers and plantation managers who need to sell their oil palm fresh fruit bunch (FFB) for the mill as this will avoid disputes. In this paper,a new approach was developed under the name of expert rules-based systembased on the image processing techniques results of thethree different oil palm FFB region of interests (ROIs), namely; ROI1 (300x300 pixels), ROI2 (50x50 pixels) and ROI3 (100x100 pixels). The results show that the best rule-based ROIs for statistical colour feature extraction with k-nearest neighbors (KNN) classifier at 94% were chosen as well as the ROIs that indicated results higher than the rule-based outcome, such as the ROIs of statistical colour feature extraction with artificial neural network (ANN) classifier at 94%, were selected for further FFB ripeness inspection system.</t>
+          <t>In this paper, a hyperspectral-based system was introduced to detect the ripeness of oil palm fresh fruit bunches (FFB). The FFBs were scanned using a hyperspectral device, and reflectance was recorded at different wavelengths. A total of 469 fruits from oil palm FFBs (nigrescens, virescens, oleifera) were categorized as overripe, ripe, and underripe. Fruit attributes in the visible and nearinfrared (400 nm to1000 nm) wavelength range regions were measured. Artificial neural network (ANN), classified the different wavelength regions on oil palm fruit through pixel-wise processing. The developed ANN model successfully classified oil palm fruits into the three ripeness categories (ripe, underripe, and overripe). The accuracy achieved by our approach was compared against that of the conventional system employing manual classification based on the observations of a human grader. Our classification approach had an accuracy of more than 95% for all three types of oil palm fruits. The research findings will help increase the quality harvesting and grading efficiency of FFBs.</t>
         </is>
       </c>
       <c r="H165" s="3" t="inlineStr">
@@ -13709,17 +13701,17 @@
       </c>
       <c r="I165" s="3" t="inlineStr">
         <is>
-          <t>KLS</t>
+          <t>SENSOR</t>
         </is>
       </c>
       <c r="J165" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>PABRIK</t>
         </is>
       </c>
       <c r="K165" s="3" t="inlineStr">
         <is>
-          <t>RGB</t>
+          <t>HSI</t>
         </is>
       </c>
       <c r="L165" s="3" t="inlineStr">
@@ -13734,10 +13726,14 @@
       </c>
       <c r="N165" s="3" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O165" s="3" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O165" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/bensaeed2014oil.txt</t>
+        </is>
+      </c>
       <c r="P165" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -13746,22 +13742,18 @@
       <c r="Q165" s="5" t="inlineStr"/>
       <c r="R165" s="5" t="inlineStr"/>
       <c r="S165" s="6" t="inlineStr"/>
-      <c r="T165" s="4" t="inlineStr">
-        <is>
-          <t>kode '?' pada: lokasi</t>
-        </is>
-      </c>
+      <c r="T165" s="4" t="inlineStr"/>
     </row>
     <row r="166" ht="110" customHeight="1">
       <c r="A166" s="3" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B166" s="3" t="n">
-        <v>2409</v>
+        <v>2410</v>
       </c>
       <c r="C166" s="3" t="inlineStr">
         <is>
-          <t>bensaeed2014oil</t>
+          <t>kassim2014oil</t>
         </is>
       </c>
       <c r="D166" s="3" t="inlineStr">
@@ -13771,17 +13763,17 @@
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>Oil palm fruit grading using a hyperspectral device and machine learning algorithm</t>
+          <t>Oil palm fruit classifications by using near infrared images</t>
         </is>
       </c>
       <c r="F166" s="3" t="inlineStr">
         <is>
-          <t>10.1088/1755-1315/20/1/012017</t>
+          <t>10.19026/rjaset.7.517</t>
         </is>
       </c>
       <c r="G166" s="4" t="inlineStr">
         <is>
-          <t>In this paper, a hyperspectral-based system was introduced to detect the ripeness of oil palm fresh fruit bunches (FFB). The FFBs were scanned using a hyperspectral device, and reflectance was recorded at different wavelengths. A total of 469 fruits from oil palm FFBs (nigrescens, virescens, oleifera) were categorized as overripe, ripe, and underripe. Fruit attributes in the visible and nearinfrared (400 nm to1000 nm) wavelength range regions were measured. Artificial neural network (ANN), classified the different wavelength regions on oil palm fruit through pixel-wise processing. The developed ANN model successfully classified oil palm fruits into the three ripeness categories (ripe, underripe, and overripe). The accuracy achieved by our approach was compared against that of the conventional system employing manual classification based on the observations of a human grader. Our classification approach had an accuracy of more than 95% for all three types of oil palm fruits. The research findings will help increase the quality harvesting and grading efficiency of FFBs.</t>
+          <t>Non-destructive assessment on oil palm Fresh Fruit Bunch (FFB) variability provides information for convenient oil palm field management practices. In this study a destructive assessment, using a microstrip sensor technique was firstly used to determine oil palm FFB maturity stages. A sample of FFB fruitlets was taken from 50 oil palm trees. The statistical data of insertion loss obtained from microstrip sensor was then been compared with moisture content in wet basis that was obtained from oven drying to correlate with the FFB maturity stages. The images of the above FFB samples were taken at the field by using multispectral camera. These images were processed and Near Infrared (NIR) hue value was extracted as the maturity feature. A relationship between images data of NIR and microstrip sensor data was developed to determine the maturity stages. The maturity stages data was plotted in the GIS map. Farmers will be able to go to specific location of FFB that has the optimum maturity and carried out the harvesting operation efficiently.</t>
         </is>
       </c>
       <c r="H166" s="3" t="inlineStr">
@@ -13796,12 +13788,12 @@
       </c>
       <c r="J166" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>POHON</t>
         </is>
       </c>
       <c r="K166" s="3" t="inlineStr">
         <is>
-          <t>HSI</t>
+          <t>MSI</t>
         </is>
       </c>
       <c r="L166" s="3" t="inlineStr">
@@ -13816,14 +13808,10 @@
       </c>
       <c r="N166" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="O166" s="3" t="inlineStr">
-        <is>
-          <t>literature/scopus-2026-09/teks/bensaeed2014oil.txt</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O166" s="3" t="inlineStr"/>
       <c r="P166" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -13832,22 +13820,18 @@
       <c r="Q166" s="5" t="inlineStr"/>
       <c r="R166" s="5" t="inlineStr"/>
       <c r="S166" s="6" t="inlineStr"/>
-      <c r="T166" s="4" t="inlineStr">
-        <is>
-          <t>kode '?' pada: lokasi</t>
-        </is>
-      </c>
+      <c r="T166" s="4" t="inlineStr"/>
     </row>
     <row r="167" ht="110" customHeight="1">
       <c r="A167" s="3" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B167" s="3" t="n">
-        <v>2410</v>
+        <v>2391</v>
       </c>
       <c r="C167" s="3" t="inlineStr">
         <is>
-          <t>kassim2014oil</t>
+          <t>makky2014automatic</t>
         </is>
       </c>
       <c r="D167" s="3" t="inlineStr">
@@ -13857,17 +13841,17 @@
       </c>
       <c r="E167" s="4" t="inlineStr">
         <is>
-          <t>Oil palm fruit classifications by using near infrared images</t>
+          <t>Automatic non-destructive quality inspection system for oil palm fruits</t>
         </is>
       </c>
       <c r="F167" s="3" t="inlineStr">
         <is>
-          <t>10.19026/rjaset.7.517</t>
+          <t>10.2478/intag-2014-0022</t>
         </is>
       </c>
       <c r="G167" s="4" t="inlineStr">
         <is>
-          <t>Non-destructive assessment on oil palm Fresh Fruit Bunch (FFB) variability provides information for convenient oil palm field management practices. In this study a destructive assessment, using a microstrip sensor technique was firstly used to determine oil palm FFB maturity stages. A sample of FFB fruitlets was taken from 50 oil palm trees. The statistical data of insertion loss obtained from microstrip sensor was then been compared with moisture content in wet basis that was obtained from oven drying to correlate with the FFB maturity stages. The images of the above FFB samples were taken at the field by using multispectral camera. These images were processed and Near Infrared (NIR) hue value was extracted as the maturity feature. A relationship between images data of NIR and microstrip sensor data was developed to determine the maturity stages. The maturity stages data was plotted in the GIS map. Farmers will be able to go to specific location of FFB that has the optimum maturity and carried out the harvesting operation efficiently.</t>
+          <t>Abstract In this research a non-destructive, rapid and cost effective examination machine for the estimation of the ripeness fraction, oil content and free fatty acid level in oil palm fresh fruits bunch was developed. The automatic machine-vision based inspection system provided consistency, rapid estimation and acceptable accuracy results in non-destructive manner. Fresh fruits bunch samples from Tenera cultivar (7 to 20 years trees) were taken from Cimulang plantation, Bogor, Indonesia. Two statistical analysis methods were used: a forward stepwise multiple linear regression analysis and a multilayer-perceptron artificial neural network analysis. The best prediction of ripeness and oil content models were obtained using the latter method, while the best free fatty acid prediction model was developed by the first method. The models were then employed in the machine-vision inspection systems of the machine. The system best prediction accuracy of ripeness, oil content and free fatty acid models was 93.5, 96.41, and 89.32%, with standard error of prediction being 0.065, 0.044 and 0.068, respectively. The system was tested through a series of field tests, and successfully examined more than 12 t of fruits bunch per hour, without causing damage.</t>
         </is>
       </c>
       <c r="H167" s="3" t="inlineStr">
@@ -13877,17 +13861,17 @@
       </c>
       <c r="I167" s="3" t="inlineStr">
         <is>
-          <t>SENSOR</t>
+          <t>MUTU</t>
         </is>
       </c>
       <c r="J167" s="3" t="inlineStr">
         <is>
-          <t>POHON</t>
+          <t>PABRIK</t>
         </is>
       </c>
       <c r="K167" s="3" t="inlineStr">
         <is>
-          <t>MSI</t>
+          <t>RGB</t>
         </is>
       </c>
       <c r="L167" s="3" t="inlineStr">
@@ -13902,10 +13886,14 @@
       </c>
       <c r="N167" s="3" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O167" s="3" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O167" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/makky2014automatic.txt</t>
+        </is>
+      </c>
       <c r="P167" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -13918,34 +13906,34 @@
     </row>
     <row r="168" ht="110" customHeight="1">
       <c r="A168" s="3" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B168" s="3" t="n">
-        <v>2391</v>
+        <v>2450</v>
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>makky2014automatic</t>
+          <t>makky2013development</t>
         </is>
       </c>
       <c r="D168" s="3" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>Automatic non-destructive quality inspection system for oil palm fruits</t>
+          <t>Development of an automatic grading machine for oil palm fresh fruits bunches (FFBs) based on machine vision</t>
         </is>
       </c>
       <c r="F168" s="3" t="inlineStr">
         <is>
-          <t>10.2478/intag-2014-0022</t>
+          <t>10.1016/j.compag.2013.02.008</t>
         </is>
       </c>
       <c r="G168" s="4" t="inlineStr">
         <is>
-          <t>Abstract In this research a non-destructive, rapid and cost effective examination machine for the estimation of the ripeness fraction, oil content and free fatty acid level in oil palm fresh fruits bunch was developed. The automatic machine-vision based inspection system provided consistency, rapid estimation and acceptable accuracy results in non-destructive manner. Fresh fruits bunch samples from Tenera cultivar (7 to 20 years trees) were taken from Cimulang plantation, Bogor, Indonesia. Two statistical analysis methods were used: a forward stepwise multiple linear regression analysis and a multilayer-perceptron artificial neural network analysis. The best prediction of ripeness and oil content models were obtained using the latter method, while the best free fatty acid prediction model was developed by the first method. The models were then employed in the machine-vision inspection systems of the machine. The system best prediction accuracy of ripeness, oil content and free fatty acid models was 93.5, 96.41, and 89.32%, with standard error of prediction being 0.065, 0.044 and 0.068, respectively. The system was tested through a series of field tests, and successfully examined more than 12 t of fruits bunch per hour, without causing damage.</t>
+          <t>Despite being the main oil palm (Elaeis guineensis Jacq.) producer in the world, Indonesia still has scope to improve its productivity, which is currently limited by inconsistency in manual grading through human visual inspection. In this research, an automatic grading machine for oil palm fresh fruits bunch (FFB) is developed based on machine-vision principles of non-destructive analytical grading, using Indonesian Oil Palm Research Institute (IOPRI) standard. It is the first automatic grading machine for FFBs in Indonesia that works on-site. Machine consists of four subsystems namely mechanical, image processing, detection and controlling. The samples used were tenera variety fruit bunches from 7 to 20year old trees. Statistical analysis was performed to generate stepwise discrimination using Canonical Discriminant with Mahalanobis distance function for classifying groups, and appoint cluster center for each fraction. Results showed adaptive threshold algorithm gave 100% success rate for background removal, and texture analysis showed object of interest lies in intensity within digital number (DN) value from 100 to 200. Group classification of FFBs resulted average success rate of 93.53% with SEC of 0.4835 and SEP of 0.5165, while fraction classification had average success rate of 88.7%. Eight models are proposed to estimate weight of FFBs with average R2 of 81.39%. FFBs orientation on conveyor belt showed no influence on the sorting result, and with examination time of 1 FFB/5s, machine performs more than 12tons FFBs grading per hour.</t>
         </is>
       </c>
       <c r="H168" s="3" t="inlineStr">
@@ -13980,14 +13968,10 @@
       </c>
       <c r="N168" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="O168" s="3" t="inlineStr">
-        <is>
-          <t>literature/scopus-2026-09/teks/makky2014automatic.txt</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O168" s="3" t="inlineStr"/>
       <c r="P168" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -14000,34 +13984,34 @@
     </row>
     <row r="169" ht="110" customHeight="1">
       <c r="A169" s="3" t="n">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B169" s="3" t="n">
-        <v>2450</v>
+        <v>2468</v>
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>makky2013development</t>
+          <t>fadilah2012intelligent</t>
         </is>
       </c>
       <c r="D169" s="3" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="E169" s="4" t="inlineStr">
         <is>
-          <t>Development of an automatic grading machine for oil palm fresh fruits bunches (FFBs) based on machine vision</t>
+          <t>Intelligent color vision system for ripeness classification of oil palm fresh fruit bunch</t>
         </is>
       </c>
       <c r="F169" s="3" t="inlineStr">
         <is>
-          <t>10.1016/j.compag.2013.02.008</t>
+          <t>10.3390/s121014179</t>
         </is>
       </c>
       <c r="G169" s="4" t="inlineStr">
         <is>
-          <t>Despite being the main oil palm (Elaeis guineensis Jacq.) producer in the world, Indonesia still has scope to improve its productivity, which is currently limited by inconsistency in manual grading through human visual inspection. In this research, an automatic grading machine for oil palm fresh fruits bunch (FFB) is developed based on machine-vision principles of non-destructive analytical grading, using Indonesian Oil Palm Research Institute (IOPRI) standard. It is the first automatic grading machine for FFBs in Indonesia that works on-site. Machine consists of four subsystems namely mechanical, image processing, detection and controlling. The samples used were tenera variety fruit bunches from 7 to 20year old trees. Statistical analysis was performed to generate stepwise discrimination using Canonical Discriminant with Mahalanobis distance function for classifying groups, and appoint cluster center for each fraction. Results showed adaptive threshold algorithm gave 100% success rate for background removal, and texture analysis showed object of interest lies in intensity within digital number (DN) value from 100 to 200. Group classification of FFBs resulted average success rate of 93.53% with SEC of 0.4835 and SEP of 0.5165, while fraction classification had average success rate of 88.7%. Eight models are proposed to estimate weight of FFBs with average R2 of 81.39%. FFBs orientation on conveyor belt showed no influence on the sorting result, and with examination time of 1 FFB/5s, machine performs more than 12tons FFBs grading per hour.</t>
+          <t>Ripeness classification of oil palm fresh fruit bunches (FFBs) during harvesting is important to ensure that they are harvested during optimum stage for maximum oil production. This paper presents the application of color vision for automated ripeness classification of oil palm FFB. Images of oil palm FFBs of type DxP Yangambi were collected and analyzed using digital image processing techniques. Then the color features were extracted from those images and used as the inputs for Artificial Neural Network (ANN) learning. The performance of the ANN for ripeness classification of oil palm FFB was investigated using two methods: training ANN with full features and training ANN with reduced features based on the Principal Component Analysis (PCA) data reduction technique. Results showed that compared with using full features in ANN, using the ANN trained with reduced features can improve the classification accuracy by 1.66% and is more effective in developing an automated ripeness classifier for oil palm FFB. The developed ripeness classifier can act as a sensor in determining the correct oil palm FFB ripeness category.</t>
         </is>
       </c>
       <c r="H169" s="3" t="inlineStr">
@@ -14042,7 +14026,7 @@
       </c>
       <c r="J169" s="3" t="inlineStr">
         <is>
-          <t>PABRIK</t>
+          <t>?</t>
         </is>
       </c>
       <c r="K169" s="3" t="inlineStr">
@@ -14062,10 +14046,14 @@
       </c>
       <c r="N169" s="3" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O169" s="3" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O169" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/fadilah2012intelligent.txt</t>
+        </is>
+      </c>
       <c r="P169" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -14074,18 +14062,22 @@
       <c r="Q169" s="5" t="inlineStr"/>
       <c r="R169" s="5" t="inlineStr"/>
       <c r="S169" s="6" t="inlineStr"/>
-      <c r="T169" s="4" t="inlineStr"/>
+      <c r="T169" s="4" t="inlineStr">
+        <is>
+          <t>kode '?' pada: lokasi</t>
+        </is>
+      </c>
     </row>
     <row r="170" ht="110" customHeight="1">
       <c r="A170" s="3" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B170" s="3" t="n">
-        <v>2468</v>
+        <v>2466</v>
       </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
-          <t>fadilah2012intelligent</t>
+          <t>fadilah2012oil</t>
         </is>
       </c>
       <c r="D170" s="3" t="inlineStr">
@@ -14095,17 +14087,17 @@
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>Intelligent color vision system for ripeness classification of oil palm fresh fruit bunch</t>
+          <t>Oil palm fresh fruit bunch ripeness classification using artificial neural network</t>
         </is>
       </c>
       <c r="F170" s="3" t="inlineStr">
         <is>
-          <t>10.3390/s121014179</t>
+          <t>10.1109/icias.2012.6306151</t>
         </is>
       </c>
       <c r="G170" s="4" t="inlineStr">
         <is>
-          <t>Ripeness classification of oil palm fresh fruit bunches (FFBs) during harvesting is important to ensure that they are harvested during optimum stage for maximum oil production. This paper presents the application of color vision for automated ripeness classification of oil palm FFB. Images of oil palm FFBs of type DxP Yangambi were collected and analyzed using digital image processing techniques. Then the color features were extracted from those images and used as the inputs for Artificial Neural Network (ANN) learning. The performance of the ANN for ripeness classification of oil palm FFB was investigated using two methods: training ANN with full features and training ANN with reduced features based on the Principal Component Analysis (PCA) data reduction technique. Results showed that compared with using full features in ANN, using the ANN trained with reduced features can improve the classification accuracy by 1.66% and is more effective in developing an automated ripeness classifier for oil palm FFB. The developed ripeness classifier can act as a sensor in determining the correct oil palm FFB ripeness category.</t>
+          <t>This paper presents the ripeness classification of oil palm fresh fruit bunch (FFB) using artificial neural network (ANN). ANN method was used to automate the decision of grading oil plam FFBs, replacing the manual human grading method. A total of 80 oil palm FFB samples from unripe, underripe, ripe and overripe categories were collected. Images of oil palm FFB were obtained using a color digital camera and their color was analyzed using digital image processing techniques. Then the color features were extracted from those images. These features were used as the input parameters for ANN learning. The performance of ANN was measured by testing the network with independent test data. Results show that ANN was able to generalize four ripeness categories of oil palm FFB.</t>
         </is>
       </c>
       <c r="H170" s="3" t="inlineStr">
@@ -14140,14 +14132,10 @@
       </c>
       <c r="N170" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="O170" s="3" t="inlineStr">
-        <is>
-          <t>literature/scopus-2026-09/teks/fadilah2012intelligent.txt</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O170" s="3" t="inlineStr"/>
       <c r="P170" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -14164,34 +14152,34 @@
     </row>
     <row r="171" ht="110" customHeight="1">
       <c r="A171" s="3" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B171" s="3" t="n">
-        <v>2466</v>
+        <v>1489</v>
       </c>
       <c r="C171" s="3" t="inlineStr">
         <is>
-          <t>fadilah2012oil</t>
+          <t>syahputra2026comparative</t>
         </is>
       </c>
       <c r="D171" s="3" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E171" s="4" t="inlineStr">
         <is>
-          <t>Oil palm fresh fruit bunch ripeness classification using artificial neural network</t>
+          <t>Comparative Analysis of Oil Palm Fruit Free Fatty Acid Estimation Using a Portable VIS-NIR Spectrometer and Multispectral Imaging</t>
         </is>
       </c>
       <c r="F171" s="3" t="inlineStr">
         <is>
-          <t>10.1109/icias.2012.6306151</t>
+          <t>10.1088/1755-1315/1584/1/012033</t>
         </is>
       </c>
       <c r="G171" s="4" t="inlineStr">
         <is>
-          <t>This paper presents the ripeness classification of oil palm fresh fruit bunch (FFB) using artificial neural network (ANN). ANN method was used to automate the decision of grading oil plam FFBs, replacing the manual human grading method. A total of 80 oil palm FFB samples from unripe, underripe, ripe and overripe categories were collected. Images of oil palm FFB were obtained using a color digital camera and their color was analyzed using digital image processing techniques. Then the color features were extracted from those images. These features were used as the input parameters for ANN learning. The performance of ANN was measured by testing the network with independent test data. Results show that ANN was able to generalize four ripeness categories of oil palm FFB.</t>
+          <t>Abstract The titration method is the conventional approach for measuring free fatty acid (FFA) content in oil palm fruit but is destructive and time-consuming. Since FFA is a critical quality parameter in Indonesia’s palm oil industry, there is an urgent need for rapid, non-destructive alternatives. This study presents a comparative analysis of two non-invasive sensing technologies for estimating oil palm FFA: a portable visible–near infrared (VIS-NIR) spectrometer and a multispectral imaging system. Fruit samples at various maturity stages were analyzed using both methods. The VIS-NIR spectrometer captured spectral reIlectance in the red band (660–670 nm), while the multispectral camera provided corresponding image intensity features. Principal Component Analysis (PCA) of the red band reIlectance showed that PC1 accounted for 98.47% of the variance, clearly separating all ripeness classes. Regression analysis conIirmed strong correlations with FFA content, with the VIS-NIR spectrometer achieving R 2 = 0.85 and multispectral imaging R 2 = 0.79. Expanding the dataset across multiple cultivars and environmental conditions, combined with advanced multivariate modeling, could further improve prediction accuracy. These Iindings demonstrate that both technologies can provide accurate, rapid, and non-destructive estimation of FFA, supporting real-time quality monitoring and improved harvest management in Indonesia’s palm oil sector.</t>
         </is>
       </c>
       <c r="H171" s="3" t="inlineStr">
@@ -14201,7 +14189,7 @@
       </c>
       <c r="I171" s="3" t="inlineStr">
         <is>
-          <t>KLS</t>
+          <t>MUTU</t>
         </is>
       </c>
       <c r="J171" s="3" t="inlineStr">
@@ -14211,7 +14199,7 @@
       </c>
       <c r="K171" s="3" t="inlineStr">
         <is>
-          <t>RGB</t>
+          <t>MSI</t>
         </is>
       </c>
       <c r="L171" s="3" t="inlineStr">
@@ -14221,7 +14209,7 @@
       </c>
       <c r="M171" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="N171" s="3" t="inlineStr">
@@ -14244,13 +14232,501 @@
         </is>
       </c>
     </row>
+    <row r="172" ht="110" customHeight="1">
+      <c r="A172" s="3" t="n">
+        <v>172</v>
+      </c>
+      <c r="B172" s="3" t="n">
+        <v>1550</v>
+      </c>
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>puttinaovarat2025innovative</t>
+        </is>
+      </c>
+      <c r="D172" s="3" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E172" s="4" t="inlineStr">
+        <is>
+          <t>Innovative Flood Impact Monitoring and Harvest Analysis in Oil Palm Plantations Utilizing Geographic Information Systems and Deep Learning</t>
+        </is>
+      </c>
+      <c r="F172" s="3" t="inlineStr">
+        <is>
+          <t>10.3390/agriengineering7020044</t>
+        </is>
+      </c>
+      <c r="G172" s="4" t="inlineStr">
+        <is>
+          <t>Floods, as a form of disaster, significantly affect individuals and farmers in impacted areas, particularly through crop damage and the inability to harvest due to prolonged and extensive flooding. Among the most severely affected agricultural sectors are oil palm plantations, which regularly experience such disruptions annually. Current methods of assistance and relief during flooding rely on field surveys conducted manually by personnel, a process constrained by its time-intensive nature. Moreover, existing applications or platforms do not support the classification and inspection of oil palm plantations affected by floods during harvesting. This research aims to develop a method and application for inspecting oil palm plantations impacted by floods during harvesting. The approach utilizes deep learning and geographic information systems (GIS) to classify and analyze flood-affected areas and determine the ripeness of oil palm bunches on trees, enabling accurate and rapid identification of flood-affected areas. The study results demonstrate that the proposed method achieves a flood classification accuracy ranging from 96.80% to 98.29% and ripeness classification accuracy for oil palm bunches on trees ranging from 97.60% to 99.75%. These findings indicate that the proposed model effectively and efficiently monitors flood-affected areas. Additionally, the developed application serves as a valuable tool for flood management, facilitating timely assistance and relief for farmers impacted by flooding.</t>
+        </is>
+      </c>
+      <c r="H172" s="3" t="inlineStr">
+        <is>
+          <t>abstrak</t>
+        </is>
+      </c>
+      <c r="I172" s="3" t="inlineStr">
+        <is>
+          <t>KLS</t>
+        </is>
+      </c>
+      <c r="J172" s="3" t="inlineStr">
+        <is>
+          <t>POHON</t>
+        </is>
+      </c>
+      <c r="K172" s="3" t="inlineStr">
+        <is>
+          <t>RGB</t>
+        </is>
+      </c>
+      <c r="L172" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M172" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N172" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O172" s="3" t="inlineStr"/>
+      <c r="P172" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q172" s="5" t="inlineStr"/>
+      <c r="R172" s="5" t="inlineStr"/>
+      <c r="S172" s="6" t="inlineStr"/>
+      <c r="T172" s="4" t="inlineStr"/>
+    </row>
+    <row r="173" ht="110" customHeight="1">
+      <c r="A173" s="3" t="n">
+        <v>173</v>
+      </c>
+      <c r="B173" s="3" t="n">
+        <v>1767</v>
+      </c>
+      <c r="C173" s="3" t="inlineStr">
+        <is>
+          <t>phimpisan2023real</t>
+        </is>
+      </c>
+      <c r="D173" s="3" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E173" s="4" t="inlineStr">
+        <is>
+          <t>Real-Time oil palm ripeness classification of fresh fruit bunches using fluorescence technology</t>
+        </is>
+      </c>
+      <c r="F173" s="3" t="inlineStr">
+        <is>
+          <t>10.34044/j.anres.2023.57.5.12</t>
+        </is>
+      </c>
+      <c r="G173" s="4" t="inlineStr">
+        <is>
+          <t>Importance of the work: The precise and non-destructive grading of oil palm fresh fruit bunches (OPFFBs) is crucial in determining the profit for farmers selling the product to factories.Objectives: To investigate the accuracy of fluorescence technology combined with image analysis technology in categorizing OPFFB ripeness. Materials &amp; Methods:A combination of eight ultraviolet light-emitting diodes (UV LEDs) were used in the wavelength range 395-400 nm along with image processing techniques to classify oil palm ripening in the Tenera variety (80 ripe and 20 under-ripe bunches).Afterward, the UV LEDs stimulated the OPFFBs in darkness, as indicated by fluorescence in the image processing.To validate the results, the fluorescence visibility results were compared with the results manually provided by five experts and with crude palm oil percentages obtained from 600 fruits samples extracted using an organic solvent (six fruits were sampled from each bunch).Results: The equipment yielded results that were deemed 100% accurate, as confirmed by experts and the crude palm oil percentages obtained from laboratory analysis. Main finding:The research equipment demonstrated enhanced fluorescence visibility for assessing the maturity of Tenera variety oil palm fresh fruit bunches.This technique may have potential applications in assessing the maturity of other oil palm varieties, as well as different types of fruit.</t>
+        </is>
+      </c>
+      <c r="H173" s="3" t="inlineStr">
+        <is>
+          <t>abstrak</t>
+        </is>
+      </c>
+      <c r="I173" s="3" t="inlineStr">
+        <is>
+          <t>KLS</t>
+        </is>
+      </c>
+      <c r="J173" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="K173" s="3" t="inlineStr">
+        <is>
+          <t>RGB</t>
+        </is>
+      </c>
+      <c r="L173" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M173" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N173" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O173" s="3" t="inlineStr"/>
+      <c r="P173" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q173" s="5" t="inlineStr"/>
+      <c r="R173" s="5" t="inlineStr"/>
+      <c r="S173" s="6" t="inlineStr"/>
+      <c r="T173" s="4" t="inlineStr">
+        <is>
+          <t>kode '?' pada: lokasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" ht="110" customHeight="1">
+      <c r="A174" s="3" t="n">
+        <v>174</v>
+      </c>
+      <c r="B174" s="3" t="n">
+        <v>1991</v>
+      </c>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>melidawati2021non</t>
+        </is>
+      </c>
+      <c r="D174" s="3" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="E174" s="4" t="inlineStr">
+        <is>
+          <t>Non destructive evaluation quality of oil palm fresh fruit bunch (FFB) (Elaeis guineensis Jack) based on optical properties using artificial neural network (ANN)</t>
+        </is>
+      </c>
+      <c r="F174" s="3" t="inlineStr">
+        <is>
+          <t>10.1088/1755-1315/644/1/012032</t>
+        </is>
+      </c>
+      <c r="G174" s="4" t="inlineStr">
+        <is>
+          <t>Abstract Oil palm (Elaeis guineensis Jacq) is one of the oil-producing plants with high productivity. The quality of palm fresh fruit bunches (FFB) is affected by harvesting activities. Generally, the method of harvesting oil palm by visual observation (maturity fraction) and harvest rotation systems. This study evaluated the quality of oil palm FFB non-destructively based on optical properties. Oil palm Fresh Fruit Bunches harvested in 5 ripeness ranges (110-130 DAA, 131-150 DAA, 151-170 DAA, 171-190 DAA, and 191-200 DAA). The oil palm FFB image recorded using a mobile camera with a minimum resolution of 25 megapixels, and then the image was processed using a digital image processing program. Furthermore, the quality parameters of oil palm FFB tested, and data were analyzed using SPSS Statistics 20.0 with the Artificial Neural Network (ANN) method. The model’s R2 upon calibration was 0.6934. While upon validation R2 value was 0.7211. The model was considered appropriate since R2 value both in calibration and validation were high.</t>
+        </is>
+      </c>
+      <c r="H174" s="3" t="inlineStr">
+        <is>
+          <t>abstrak</t>
+        </is>
+      </c>
+      <c r="I174" s="3" t="inlineStr">
+        <is>
+          <t>MUTU</t>
+        </is>
+      </c>
+      <c r="J174" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="K174" s="3" t="inlineStr">
+        <is>
+          <t>RGB</t>
+        </is>
+      </c>
+      <c r="L174" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M174" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N174" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O174" s="3" t="inlineStr"/>
+      <c r="P174" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q174" s="5" t="inlineStr"/>
+      <c r="R174" s="5" t="inlineStr"/>
+      <c r="S174" s="6" t="inlineStr"/>
+      <c r="T174" s="4" t="inlineStr">
+        <is>
+          <t>kode '?' pada: lokasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" ht="110" customHeight="1">
+      <c r="A175" s="3" t="n">
+        <v>175</v>
+      </c>
+      <c r="B175" s="3" t="n">
+        <v>2078</v>
+      </c>
+      <c r="C175" s="3" t="inlineStr">
+        <is>
+          <t>aliteh2020fruit</t>
+        </is>
+      </c>
+      <c r="D175" s="3" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="E175" s="4" t="inlineStr">
+        <is>
+          <t>Fruit battery method for oil palm fruit ripeness sensor and comparison with computer vision method</t>
+        </is>
+      </c>
+      <c r="F175" s="3" t="inlineStr">
+        <is>
+          <t>10.3390/s20030637</t>
+        </is>
+      </c>
+      <c r="G175" s="4" t="inlineStr">
+        <is>
+          <t>Oil palm ripeness' main evaluation procedure is traditionally accomplished by human vision. However, the dependency on human evaluators to grade the ripeness of oil palm fresh fruit bunches (FFBs) by traditional means could lead to inaccuracy that can cause a reduction in oil palm fruit oil extraction rate (OER). This paper emphasizes the fruit battery method to distinguish oil palm fruit FFB ripeness stages by determining the value of load resistance voltage and its moisture content resolution. In addition, computer vision using a color feature is tested on the same samples to compare the accuracy score using support vector machine (SVM). The accuracy score results of the fruit battery, computer vision, and a combination of both methods' accuracy scores are evaluated and compared. When the ripe and unripe samples were tested for load resistance voltage ranging from 10 Ω to 10 kΩ, three resistance values were shortlisted and tested for moisture content resolution evaluation. A 1 kΩ load resistance showed the best moisture content resolution, and the results were used for accuracy score evaluation comparison with computer vision. From the results obtained, the accuracy scores for the combination method are the highest, followed by the fruit battery and computer vision methods.</t>
+        </is>
+      </c>
+      <c r="H175" s="3" t="inlineStr">
+        <is>
+          <t>abstrak</t>
+        </is>
+      </c>
+      <c r="I175" s="3" t="inlineStr">
+        <is>
+          <t>KLS</t>
+        </is>
+      </c>
+      <c r="J175" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="K175" s="3" t="inlineStr">
+        <is>
+          <t>RGB</t>
+        </is>
+      </c>
+      <c r="L175" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M175" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N175" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O175" s="3" t="inlineStr"/>
+      <c r="P175" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q175" s="5" t="inlineStr"/>
+      <c r="R175" s="5" t="inlineStr"/>
+      <c r="S175" s="6" t="inlineStr"/>
+      <c r="T175" s="4" t="inlineStr">
+        <is>
+          <t>kode '?' pada: lokasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" ht="110" customHeight="1">
+      <c r="A176" s="3" t="n">
+        <v>176</v>
+      </c>
+      <c r="B176" s="3" t="n">
+        <v>2368</v>
+      </c>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>cherie2015optical</t>
+        </is>
+      </c>
+      <c r="D176" s="3" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="E176" s="4" t="inlineStr">
+        <is>
+          <t>Optical characteristics of oil palm fresh fruits bunch (FFB) under three spectrum regions influence for harvest decision</t>
+        </is>
+      </c>
+      <c r="F176" s="3" t="inlineStr">
+        <is>
+          <t>10.18517/ijaseit.5.3.534</t>
+        </is>
+      </c>
+      <c r="G176" s="4" t="inlineStr">
+        <is>
+          <t>In current practice, appearance was used to determine ripeness for oil palm fresh fruits bunch (FFB), that accompanied by detachment of fruit-lets from the bunch. The FFB from marihat clone harvested at five ripeness stages, under ripeness (F0), ripeness (F1, F2, F3), and over ripeness (F4). At every ripeness stages, differences of oil content and pigment accumulation were observed on the bunch. All samples recorded using a digital camera (10 Mpixel) from 2, 7, 10, and 15 meter distance, simulating variation of light intensity upon recording. During image recording, three lighting were used, namely ultraviolet lamp (320-380 nm), visible light lamp (400-700 nm) and infrared lamp (720-1100 nm), all have similar power output of 600watt. Camera point of view was set to cover a square area of 12,5cm by 12,5cm of the frontal area of FFB, each picture produced has 3888 by 2952 pixel. Image processing software created to extract digital RGB information from the images, and displayed the information in histogram. From the experiment, it was observed that the changes of intensity influence the RGB value of recorded image with reverse correlation, and longer wave light spectrum produce smaller RGB value. The correlation model among image recording distance and RGB of the image display similar nature. From three color channels, G represents better correlation for sample’s oil content determination. Using UV and visible lighting, the FFB samples may be determined for harvest decision, up to seven meter observation distance.</t>
+        </is>
+      </c>
+      <c r="H176" s="3" t="inlineStr">
+        <is>
+          <t>abstrak</t>
+        </is>
+      </c>
+      <c r="I176" s="3" t="inlineStr">
+        <is>
+          <t>SENSOR</t>
+        </is>
+      </c>
+      <c r="J176" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="K176" s="3" t="inlineStr">
+        <is>
+          <t>RGB</t>
+        </is>
+      </c>
+      <c r="L176" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M176" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N176" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O176" s="3" t="inlineStr"/>
+      <c r="P176" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q176" s="5" t="inlineStr"/>
+      <c r="R176" s="5" t="inlineStr"/>
+      <c r="S176" s="6" t="inlineStr"/>
+      <c r="T176" s="4" t="inlineStr">
+        <is>
+          <t>kode '?' pada: lokasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" ht="110" customHeight="1">
+      <c r="A177" s="3" t="n">
+        <v>177</v>
+      </c>
+      <c r="B177" s="3" t="n">
+        <v>2486</v>
+      </c>
+      <c r="C177" s="3" t="inlineStr">
+        <is>
+          <t>hudzari2012simulation</t>
+        </is>
+      </c>
+      <c r="D177" s="3" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="E177" s="4" t="inlineStr">
+        <is>
+          <t>Simulation and modeling application in agricultural mechanization</t>
+        </is>
+      </c>
+      <c r="F177" s="3" t="inlineStr">
+        <is>
+          <t>10.1155/2012/381239</t>
+        </is>
+      </c>
+      <c r="G177" s="4" t="inlineStr">
+        <is>
+          <t>This experiment was conducted to determine the equations relating the Hue digital values of the fruits surface of the oil palm with maturity stage of the fruit in plantation. The FFB images were zoomed and captured using Nikon digital camera, and the calculation of Hue was determined using the highest frequency of the value forR,G, andBcolor components from histogram analysis software. New procedure in monitoring the image pixel value for oil palm fruit color surface in real-time growth maturity was developed. The estimation of day harvesting prediction was calculated based on developed model of relationships for Hue values with mesocarp oil content. The simulation model is regressed and predicts the day of harvesting or a number of days before harvest of FFB. The result from experimenting on mesocarp oil content can be used for real-time oil content determination of MPOB color meter. The graph to determine the day of harvesting the FFB was presented in this research. The oil was found to start developing in mesocarp fruit at 65 days before fruit at ripe maturity stage of 75% oil to dry mesocarp.</t>
+        </is>
+      </c>
+      <c r="H177" s="3" t="inlineStr">
+        <is>
+          <t>abstrak</t>
+        </is>
+      </c>
+      <c r="I177" s="3" t="inlineStr">
+        <is>
+          <t>KLS</t>
+        </is>
+      </c>
+      <c r="J177" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="K177" s="3" t="inlineStr">
+        <is>
+          <t>RGB</t>
+        </is>
+      </c>
+      <c r="L177" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M177" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N177" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O177" s="3" t="inlineStr"/>
+      <c r="P177" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q177" s="5" t="inlineStr"/>
+      <c r="R177" s="5" t="inlineStr"/>
+      <c r="S177" s="6" t="inlineStr"/>
+      <c r="T177" s="4" t="inlineStr">
+        <is>
+          <t>kode '?' pada: lokasi</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T171"/>
+  <autoFilter ref="A1:T177"/>
   <dataValidations count="2">
-    <dataValidation sqref="Q2:Q371" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Pilih salah satu: Y,N" type="list">
+    <dataValidation sqref="Q2:Q377" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Pilih salah satu: Y,N" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
-    <dataValidation sqref="R2:R371" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Pilih salah satu: Y,N" type="list">
+    <dataValidation sqref="R2:R377" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Pilih salah satu: Y,N" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Cek 2, 5, 6: isikan usul model yang siap ke lembar; draf Cek 3, 5, 6 dan sisa Cek 2
Isian berasal dari model dan ditandai demikian di kolom catatan; belum dibaca peninjau.
- Cek 2: cek_C3 165 lengkap + 7 konfirmasi, cek_eksklusi 132
- Cek 5: 147 baris final_* (kode tidak berubah); draf_ai_* diperbarui untuk 190 kajian
- Cek 6: 263 dari 273 klaim
Sisa keputusan peninjau tercatat di hasil-kerja-ai/PERLU-DICEK.md.
</commit_message>
<xml_diff>
--- a/literature/scopus-2026-09/verifikasi/cek-2-cek-tangan/cek_C3.xlsx
+++ b/literature/scopus-2026-09/verifikasi/cek-2-cek-tangan/cek_C3.xlsx
@@ -644,9 +644,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q2" s="5" t="inlineStr"/>
-      <c r="R2" s="5" t="inlineStr"/>
-      <c r="S2" s="6" t="inlineStr"/>
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R2" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S2" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak dari web. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T2" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI</t>
@@ -718,9 +730,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q3" s="5" t="inlineStr"/>
-      <c r="R3" s="5" t="inlineStr"/>
-      <c r="S3" s="6" t="inlineStr"/>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S3" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: judul saja. Usul koreksi kode: lokasi POHON menjadi ?. Kolom yang tidak pasti menurut penilai: lokasi,modalitas,multipandang,per_kelas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T3" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI</t>
@@ -796,9 +820,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr"/>
-      <c r="R4" s="5" t="inlineStr"/>
-      <c r="S4" s="6" t="inlineStr"/>
+      <c r="Q4" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S4" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian ulang Sonnet 5.5 (satu penilai, tanpa pemeriksa). Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: judul saja. Bukti tidak cukup untuk memutuskan (tebakan: C3). Penilaian ulang Sonnet 5.5, 13 Oktober 2026, dari abstrak: C3, kode rinci sama dengan kode lembar. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T4" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
@@ -878,9 +914,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q5" s="5" t="inlineStr"/>
-      <c r="R5" s="5" t="inlineStr"/>
-      <c r="S5" s="6" t="inlineStr"/>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R5" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S5" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T5" s="4" t="inlineStr"/>
     </row>
     <row r="6" ht="110" customHeight="1">
@@ -952,9 +1000,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q6" s="5" t="inlineStr"/>
-      <c r="R6" s="5" t="inlineStr"/>
-      <c r="S6" s="6" t="inlineStr"/>
+      <c r="Q6" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R6" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S6" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T6" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
@@ -1030,9 +1090,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q7" s="5" t="inlineStr"/>
-      <c r="R7" s="5" t="inlineStr"/>
-      <c r="S7" s="6" t="inlineStr"/>
+      <c r="Q7" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R7" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S7" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian ulang Sonnet 5.5 (satu penilai, tanpa pemeriksa). Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: judul saja. Bukti tidak cukup untuk memutuskan (tebakan: X E5). Penilaian ulang Sonnet 5.5, 13 Oktober 2026, dari abstrak: C3, kode rinci sama dengan kode lembar. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T7" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
@@ -1186,9 +1258,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q9" s="5" t="inlineStr"/>
-      <c r="R9" s="5" t="inlineStr"/>
-      <c r="S9" s="6" t="inlineStr"/>
+      <c r="Q9" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R9" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S9" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T9" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
@@ -1264,9 +1348,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q10" s="5" t="inlineStr"/>
-      <c r="R10" s="5" t="inlineStr"/>
-      <c r="S10" s="6" t="inlineStr"/>
+      <c r="Q10" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R10" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S10" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: judul saja.  Kolom yang tidak pasti menurut penilai: lokasi,modalitas,multipandang,per_kelas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T10" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
@@ -1342,9 +1438,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q11" s="5" t="inlineStr"/>
-      <c r="R11" s="5" t="inlineStr"/>
-      <c r="S11" s="6" t="inlineStr"/>
+      <c r="Q11" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S11" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T11" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI</t>
@@ -1502,9 +1610,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q13" s="5" t="inlineStr"/>
+      <c r="Q13" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="R13" s="5" t="inlineStr"/>
-      <c r="S13" s="6" t="inlineStr"/>
+      <c r="S13" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: teks lengkap. Bukan C3; usul kode X E6. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -1580,9 +1696,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q14" s="5" t="inlineStr"/>
-      <c r="R14" s="5" t="inlineStr"/>
-      <c r="S14" s="6" t="inlineStr"/>
+      <c r="Q14" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R14" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S14" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: judul saja.  Kolom yang tidak pasti menurut penilai: lokasi,modalitas,multipandang. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T14" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
@@ -1658,9 +1786,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q15" s="5" t="inlineStr"/>
-      <c r="R15" s="5" t="inlineStr"/>
-      <c r="S15" s="6" t="inlineStr"/>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S15" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: judul saja.  Kolom yang tidak pasti menurut penilai: lokasi,modalitas,multipandang,per_kelas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
@@ -1736,9 +1876,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q16" s="5" t="inlineStr"/>
+      <c r="Q16" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="R16" s="5" t="inlineStr"/>
-      <c r="S16" s="6" t="inlineStr"/>
+      <c r="S16" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: teks lengkap. Bukan C3; usul kode C1. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T16" s="4" t="inlineStr"/>
     </row>
     <row r="17" ht="110" customHeight="1">
@@ -1814,9 +1962,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q17" s="5" t="inlineStr"/>
-      <c r="R17" s="5" t="inlineStr"/>
-      <c r="S17" s="6" t="inlineStr"/>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R17" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S17" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -1892,9 +2052,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q18" s="5" t="inlineStr"/>
-      <c r="R18" s="5" t="inlineStr"/>
-      <c r="S18" s="6" t="inlineStr"/>
+      <c r="Q18" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R18" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S18" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T18" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
@@ -1970,9 +2142,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q19" s="5" t="inlineStr"/>
-      <c r="R19" s="5" t="inlineStr"/>
-      <c r="S19" s="6" t="inlineStr"/>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R19" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S19" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
@@ -2048,9 +2232,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q20" s="5" t="inlineStr"/>
-      <c r="R20" s="5" t="inlineStr"/>
-      <c r="S20" s="6" t="inlineStr"/>
+      <c r="Q20" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R20" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S20" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T20" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
@@ -2126,9 +2322,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q21" s="5" t="inlineStr"/>
-      <c r="R21" s="5" t="inlineStr"/>
-      <c r="S21" s="6" t="inlineStr"/>
+      <c r="Q21" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R21" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S21" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
@@ -2278,9 +2486,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q23" s="5" t="inlineStr"/>
-      <c r="R23" s="5" t="inlineStr"/>
-      <c r="S23" s="6" t="inlineStr"/>
+      <c r="Q23" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R23" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S23" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI</t>
@@ -2356,9 +2576,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q24" s="5" t="inlineStr"/>
-      <c r="R24" s="5" t="inlineStr"/>
-      <c r="S24" s="6" t="inlineStr"/>
+      <c r="Q24" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R24" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S24" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T24" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
@@ -2430,9 +2662,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q25" s="5" t="inlineStr"/>
-      <c r="R25" s="5" t="inlineStr"/>
-      <c r="S25" s="6" t="inlineStr"/>
+      <c r="Q25" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R25" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S25" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
@@ -2512,9 +2756,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q26" s="5" t="inlineStr"/>
-      <c r="R26" s="5" t="inlineStr"/>
-      <c r="S26" s="6" t="inlineStr"/>
+      <c r="Q26" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R26" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S26" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T26" s="4" t="inlineStr"/>
     </row>
     <row r="27" ht="110" customHeight="1">
@@ -2582,9 +2838,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q27" s="5" t="inlineStr"/>
-      <c r="R27" s="5" t="inlineStr"/>
-      <c r="S27" s="6" t="inlineStr"/>
+      <c r="Q27" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R27" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S27" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
@@ -2660,9 +2928,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q28" s="5" t="inlineStr"/>
-      <c r="R28" s="5" t="inlineStr"/>
-      <c r="S28" s="6" t="inlineStr"/>
+      <c r="Q28" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R28" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S28" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T28" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
@@ -2738,9 +3018,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q29" s="5" t="inlineStr"/>
-      <c r="R29" s="5" t="inlineStr"/>
-      <c r="S29" s="6" t="inlineStr"/>
+      <c r="Q29" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R29" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S29" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak dari web. Usul koreksi kode: per_kelas Y menjadi N. Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI</t>
@@ -2820,9 +3112,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q30" s="5" t="inlineStr"/>
-      <c r="R30" s="5" t="inlineStr"/>
-      <c r="S30" s="6" t="inlineStr"/>
+      <c r="Q30" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R30" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S30" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak dari web.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T30" s="4" t="inlineStr">
         <is>
           <t>diputuskan dari judul, tetapi abstrak kini tersedia di enrich.jsonl | kode '?' pada: lokasi</t>
@@ -2898,9 +3202,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q31" s="5" t="inlineStr"/>
-      <c r="R31" s="5" t="inlineStr"/>
-      <c r="S31" s="6" t="inlineStr"/>
+      <c r="Q31" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R31" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S31" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: judul saja.  Kolom yang tidak pasti menurut penilai: lokasi,modalitas,multipandang,per_kelas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
@@ -3054,9 +3370,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q33" s="5" t="inlineStr"/>
-      <c r="R33" s="5" t="inlineStr"/>
-      <c r="S33" s="6" t="inlineStr"/>
+      <c r="Q33" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R33" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S33" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: judul saja.  Kolom yang tidak pasti menurut penilai: tugas,lokasi,modalitas,multipandang,per_kelas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
@@ -3128,9 +3456,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q34" s="5" t="inlineStr"/>
+      <c r="Q34" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="R34" s="5" t="inlineStr"/>
-      <c r="S34" s="6" t="inlineStr"/>
+      <c r="S34" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: judul saja. Bukti tidak cukup untuk memutuskan (tebakan: C3). Penilaian ulang Sonnet 5.5, 13 Oktober 2026, dari abstrak: C3; kode rinci berbeda dari kode lembar (lokasi POHON lawan ?), belum diperiksa agen kedua. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T34" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI</t>
@@ -3206,9 +3542,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q35" s="5" t="inlineStr"/>
-      <c r="R35" s="5" t="inlineStr"/>
-      <c r="S35" s="6" t="inlineStr"/>
+      <c r="Q35" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R35" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S35" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: teks lengkap. Usul koreksi kode: per_kelas Y menjadi N. Kolom yang tidak pasti menurut penilai: tugas,per_kelas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T35" s="4" t="inlineStr"/>
     </row>
     <row r="36" ht="110" customHeight="1">
@@ -3276,9 +3624,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q36" s="5" t="inlineStr"/>
+      <c r="Q36" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="R36" s="5" t="inlineStr"/>
-      <c r="S36" s="6" t="inlineStr"/>
+      <c r="S36" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak dari web. Bukti tidak cukup untuk memutuskan (tebakan: C3). Penilaian ulang Sonnet 5.5, 13 Oktober 2026, dari abstrak: C3; kode rinci berbeda dari kode lembar (per_kelas Y lawan N), belum diperiksa agen kedua. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T36" s="4" t="inlineStr">
         <is>
           <t>tanpa abstrak dan tanpa PDF: cari abstrak/teks lengkap lewat DOI | kode '?' pada: lokasi</t>
@@ -3362,9 +3718,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q37" s="5" t="inlineStr"/>
-      <c r="R37" s="5" t="inlineStr"/>
-      <c r="S37" s="6" t="inlineStr"/>
+      <c r="Q37" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R37" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S37" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T37" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -3448,9 +3816,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q38" s="5" t="inlineStr"/>
-      <c r="R38" s="5" t="inlineStr"/>
-      <c r="S38" s="6" t="inlineStr"/>
+      <c r="Q38" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R38" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S38" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T38" s="4" t="inlineStr"/>
     </row>
     <row r="39" ht="110" customHeight="1">
@@ -3530,9 +3910,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q39" s="5" t="inlineStr"/>
-      <c r="R39" s="5" t="inlineStr"/>
-      <c r="S39" s="6" t="inlineStr"/>
+      <c r="Q39" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R39" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S39" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -3612,9 +4004,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q40" s="5" t="inlineStr"/>
-      <c r="R40" s="5" t="inlineStr"/>
-      <c r="S40" s="6" t="inlineStr"/>
+      <c r="Q40" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R40" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S40" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: lokasi POHON menjadi ?. Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T40" s="4" t="inlineStr"/>
     </row>
     <row r="41" ht="110" customHeight="1">
@@ -3694,9 +4098,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q41" s="5" t="inlineStr"/>
-      <c r="R41" s="5" t="inlineStr"/>
-      <c r="S41" s="6" t="inlineStr"/>
+      <c r="Q41" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R41" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S41" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T41" s="4" t="inlineStr"/>
     </row>
     <row r="42" ht="110" customHeight="1">
@@ -3776,9 +4192,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q42" s="5" t="inlineStr"/>
-      <c r="R42" s="5" t="inlineStr"/>
-      <c r="S42" s="6" t="inlineStr"/>
+      <c r="Q42" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R42" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S42" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T42" s="4" t="inlineStr"/>
     </row>
     <row r="43" ht="110" customHeight="1">
@@ -3858,9 +4286,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q43" s="5" t="inlineStr"/>
-      <c r="R43" s="5" t="inlineStr"/>
-      <c r="S43" s="6" t="inlineStr"/>
+      <c r="Q43" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R43" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S43" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T43" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -3944,9 +4384,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q44" s="5" t="inlineStr"/>
-      <c r="R44" s="5" t="inlineStr"/>
-      <c r="S44" s="6" t="inlineStr"/>
+      <c r="Q44" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R44" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S44" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T44" s="4" t="inlineStr"/>
     </row>
     <row r="45" ht="110" customHeight="1">
@@ -4026,9 +4478,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q45" s="5" t="inlineStr"/>
-      <c r="R45" s="5" t="inlineStr"/>
-      <c r="S45" s="6" t="inlineStr"/>
+      <c r="Q45" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R45" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S45" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T45" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -4113,9 +4577,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q46" s="5" t="inlineStr"/>
-      <c r="R46" s="5" t="inlineStr"/>
-      <c r="S46" s="6" t="inlineStr"/>
+      <c r="Q46" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R46" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S46" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T46" s="4" t="inlineStr"/>
     </row>
     <row r="47" ht="110" customHeight="1">
@@ -4191,9 +4667,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q47" s="5" t="inlineStr"/>
+      <c r="Q47" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="R47" s="5" t="inlineStr"/>
-      <c r="S47" s="6" t="inlineStr"/>
+      <c r="S47" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Penilai dan pemeriksa berbeda: tugas KLS lawan SENSOR. Kolom yang tidak pasti menurut penilai: tugas. Penilaian ulang Sonnet 5.5, 13 Oktober 2026, dari abstrak: C3; kode rinci berbeda dari kode lembar (tugas SENSOR lawan KLS; lokasi PABRIK lawan ?), belum diperiksa agen kedua. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T47" s="4" t="inlineStr"/>
     </row>
     <row r="48" ht="110" customHeight="1">
@@ -4273,9 +4757,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q48" s="5" t="inlineStr"/>
-      <c r="R48" s="5" t="inlineStr"/>
-      <c r="S48" s="6" t="inlineStr"/>
+      <c r="Q48" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R48" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S48" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T48" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -4359,9 +4855,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q49" s="5" t="inlineStr"/>
-      <c r="R49" s="5" t="inlineStr"/>
-      <c r="S49" s="6" t="inlineStr"/>
+      <c r="Q49" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R49" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S49" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T49" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -4445,9 +4953,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q50" s="5" t="inlineStr"/>
-      <c r="R50" s="5" t="inlineStr"/>
-      <c r="S50" s="6" t="inlineStr"/>
+      <c r="Q50" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R50" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S50" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T50" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -4531,9 +5051,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q51" s="5" t="inlineStr"/>
-      <c r="R51" s="5" t="inlineStr"/>
-      <c r="S51" s="6" t="inlineStr"/>
+      <c r="Q51" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R51" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S51" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T51" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -4613,9 +5145,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q52" s="5" t="inlineStr"/>
-      <c r="R52" s="5" t="inlineStr"/>
-      <c r="S52" s="6" t="inlineStr"/>
+      <c r="Q52" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S52" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: lokasi POHON menjadi ?. Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T52" s="4" t="inlineStr"/>
     </row>
     <row r="53" ht="110" customHeight="1">
@@ -4691,9 +5235,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q53" s="5" t="inlineStr"/>
-      <c r="R53" s="5" t="inlineStr"/>
-      <c r="S53" s="6" t="inlineStr"/>
+      <c r="Q53" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R53" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S53" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: lokasi POHON menjadi ?. Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T53" s="4" t="inlineStr"/>
     </row>
     <row r="54" ht="110" customHeight="1">
@@ -4769,9 +5325,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q54" s="5" t="inlineStr"/>
-      <c r="R54" s="5" t="inlineStr"/>
-      <c r="S54" s="6" t="inlineStr"/>
+      <c r="Q54" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R54" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S54" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: lokasi POHON menjadi ?. Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T54" s="4" t="inlineStr"/>
     </row>
     <row r="55" ht="110" customHeight="1">
@@ -4847,9 +5415,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q55" s="5" t="inlineStr"/>
-      <c r="R55" s="5" t="inlineStr"/>
-      <c r="S55" s="6" t="inlineStr"/>
+      <c r="Q55" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R55" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S55" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T55" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -4933,9 +5513,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q56" s="5" t="inlineStr"/>
-      <c r="R56" s="5" t="inlineStr"/>
-      <c r="S56" s="6" t="inlineStr"/>
+      <c r="Q56" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R56" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S56" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T56" s="4" t="inlineStr"/>
     </row>
     <row r="57" ht="110" customHeight="1">
@@ -5011,9 +5603,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q57" s="5" t="inlineStr"/>
-      <c r="R57" s="5" t="inlineStr"/>
-      <c r="S57" s="6" t="inlineStr"/>
+      <c r="Q57" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R57" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S57" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T57" s="4" t="inlineStr"/>
     </row>
     <row r="58" ht="110" customHeight="1">
@@ -5089,9 +5693,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q58" s="5" t="inlineStr"/>
-      <c r="R58" s="5" t="inlineStr"/>
-      <c r="S58" s="6" t="inlineStr"/>
+      <c r="Q58" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R58" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S58" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T58" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -5171,9 +5787,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q59" s="5" t="inlineStr"/>
-      <c r="R59" s="5" t="inlineStr"/>
-      <c r="S59" s="6" t="inlineStr"/>
+      <c r="Q59" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R59" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S59" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T59" s="4" t="inlineStr"/>
     </row>
     <row r="60" ht="110" customHeight="1">
@@ -5249,9 +5877,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q60" s="5" t="inlineStr"/>
-      <c r="R60" s="5" t="inlineStr"/>
-      <c r="S60" s="6" t="inlineStr"/>
+      <c r="Q60" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R60" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S60" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T60" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -5331,9 +5971,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q61" s="5" t="inlineStr"/>
-      <c r="R61" s="5" t="inlineStr"/>
-      <c r="S61" s="6" t="inlineStr"/>
+      <c r="Q61" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R61" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S61" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: lokasi POHON menjadi ?. Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T61" s="4" t="inlineStr"/>
     </row>
     <row r="62" ht="110" customHeight="1">
@@ -5413,9 +6065,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q62" s="5" t="inlineStr"/>
-      <c r="R62" s="5" t="inlineStr"/>
-      <c r="S62" s="6" t="inlineStr"/>
+      <c r="Q62" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R62" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S62" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T62" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -5499,9 +6163,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q63" s="5" t="inlineStr"/>
-      <c r="R63" s="5" t="inlineStr"/>
-      <c r="S63" s="6" t="inlineStr"/>
+      <c r="Q63" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R63" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S63" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T63" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -5581,9 +6257,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q64" s="5" t="inlineStr"/>
-      <c r="R64" s="5" t="inlineStr"/>
-      <c r="S64" s="6" t="inlineStr"/>
+      <c r="Q64" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R64" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S64" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T64" s="4" t="inlineStr"/>
     </row>
     <row r="65" ht="110" customHeight="1">
@@ -5663,9 +6351,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q65" s="5" t="inlineStr"/>
-      <c r="R65" s="5" t="inlineStr"/>
-      <c r="S65" s="6" t="inlineStr"/>
+      <c r="Q65" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R65" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S65" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T65" s="4" t="inlineStr"/>
     </row>
     <row r="66" ht="110" customHeight="1">
@@ -5745,9 +6445,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q66" s="5" t="inlineStr"/>
-      <c r="R66" s="5" t="inlineStr"/>
-      <c r="S66" s="6" t="inlineStr"/>
+      <c r="Q66" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R66" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S66" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T66" s="4" t="inlineStr"/>
     </row>
     <row r="67" ht="110" customHeight="1">
@@ -5823,9 +6535,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q67" s="5" t="inlineStr"/>
-      <c r="R67" s="5" t="inlineStr"/>
-      <c r="S67" s="6" t="inlineStr"/>
+      <c r="Q67" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R67" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S67" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T67" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -5909,9 +6633,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q68" s="5" t="inlineStr"/>
-      <c r="R68" s="5" t="inlineStr"/>
-      <c r="S68" s="6" t="inlineStr"/>
+      <c r="Q68" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R68" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S68" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T68" s="4" t="inlineStr"/>
     </row>
     <row r="69" ht="110" customHeight="1">
@@ -5987,9 +6723,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q69" s="5" t="inlineStr"/>
-      <c r="R69" s="5" t="inlineStr"/>
-      <c r="S69" s="6" t="inlineStr"/>
+      <c r="Q69" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R69" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S69" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: lokasi POHON menjadi ?. Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T69" s="4" t="inlineStr"/>
     </row>
     <row r="70" ht="110" customHeight="1">
@@ -6065,9 +6813,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q70" s="5" t="inlineStr"/>
-      <c r="R70" s="5" t="inlineStr"/>
-      <c r="S70" s="6" t="inlineStr"/>
+      <c r="Q70" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R70" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S70" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T70" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -6147,9 +6907,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q71" s="5" t="inlineStr"/>
-      <c r="R71" s="5" t="inlineStr"/>
-      <c r="S71" s="6" t="inlineStr"/>
+      <c r="Q71" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R71" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S71" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T71" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -6229,9 +7001,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q72" s="5" t="inlineStr"/>
-      <c r="R72" s="5" t="inlineStr"/>
-      <c r="S72" s="6" t="inlineStr"/>
+      <c r="Q72" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R72" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S72" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T72" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -6311,9 +7095,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q73" s="5" t="inlineStr"/>
-      <c r="R73" s="5" t="inlineStr"/>
-      <c r="S73" s="6" t="inlineStr"/>
+      <c r="Q73" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R73" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S73" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi,tugas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T73" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -6397,9 +7193,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q74" s="5" t="inlineStr"/>
-      <c r="R74" s="5" t="inlineStr"/>
-      <c r="S74" s="6" t="inlineStr"/>
+      <c r="Q74" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R74" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S74" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T74" s="4" t="inlineStr"/>
     </row>
     <row r="75" ht="110" customHeight="1">
@@ -6475,9 +7283,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q75" s="5" t="inlineStr"/>
-      <c r="R75" s="5" t="inlineStr"/>
-      <c r="S75" s="6" t="inlineStr"/>
+      <c r="Q75" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R75" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S75" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T75" s="4" t="inlineStr"/>
     </row>
     <row r="76" ht="110" customHeight="1">
@@ -6553,9 +7373,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q76" s="5" t="inlineStr"/>
-      <c r="R76" s="5" t="inlineStr"/>
-      <c r="S76" s="6" t="inlineStr"/>
+      <c r="Q76" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R76" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S76" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: lokasi POHON menjadi ?. Kolom yang tidak pasti menurut penilai: tugas,lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T76" s="4" t="inlineStr"/>
     </row>
     <row r="77" ht="110" customHeight="1">
@@ -6631,9 +7463,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q77" s="5" t="inlineStr"/>
-      <c r="R77" s="5" t="inlineStr"/>
-      <c r="S77" s="6" t="inlineStr"/>
+      <c r="Q77" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R77" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S77" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T77" s="4" t="inlineStr"/>
     </row>
     <row r="78" ht="110" customHeight="1">
@@ -6709,9 +7553,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q78" s="5" t="inlineStr"/>
-      <c r="R78" s="5" t="inlineStr"/>
-      <c r="S78" s="6" t="inlineStr"/>
+      <c r="Q78" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R78" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S78" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T78" s="4" t="inlineStr"/>
     </row>
     <row r="79" ht="110" customHeight="1">
@@ -6787,9 +7643,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q79" s="5" t="inlineStr"/>
-      <c r="R79" s="5" t="inlineStr"/>
-      <c r="S79" s="6" t="inlineStr"/>
+      <c r="Q79" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R79" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S79" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: per_kelas Y menjadi N. Kolom yang tidak pasti menurut penilai: per_kelas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T79" s="4" t="inlineStr"/>
     </row>
     <row r="80" ht="110" customHeight="1">
@@ -6865,9 +7733,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q80" s="5" t="inlineStr"/>
-      <c r="R80" s="5" t="inlineStr"/>
-      <c r="S80" s="6" t="inlineStr"/>
+      <c r="Q80" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R80" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S80" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T80" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -6947,9 +7827,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q81" s="5" t="inlineStr"/>
-      <c r="R81" s="5" t="inlineStr"/>
-      <c r="S81" s="6" t="inlineStr"/>
+      <c r="Q81" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R81" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S81" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T81" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -7029,9 +7921,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q82" s="5" t="inlineStr"/>
-      <c r="R82" s="5" t="inlineStr"/>
-      <c r="S82" s="6" t="inlineStr"/>
+      <c r="Q82" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R82" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S82" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T82" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -7111,9 +8015,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q83" s="5" t="inlineStr"/>
-      <c r="R83" s="5" t="inlineStr"/>
-      <c r="S83" s="6" t="inlineStr"/>
+      <c r="Q83" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R83" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S83" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T83" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -7197,9 +8113,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q84" s="5" t="inlineStr"/>
-      <c r="R84" s="5" t="inlineStr"/>
-      <c r="S84" s="6" t="inlineStr"/>
+      <c r="Q84" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R84" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S84" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T84" s="4" t="inlineStr"/>
     </row>
     <row r="85" ht="110" customHeight="1">
@@ -7279,9 +8207,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q85" s="5" t="inlineStr"/>
-      <c r="R85" s="5" t="inlineStr"/>
-      <c r="S85" s="6" t="inlineStr"/>
+      <c r="Q85" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R85" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S85" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T85" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -7361,9 +8301,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q86" s="5" t="inlineStr"/>
-      <c r="R86" s="5" t="inlineStr"/>
-      <c r="S86" s="6" t="inlineStr"/>
+      <c r="Q86" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R86" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S86" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi,per_kelas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T86" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -7443,9 +8395,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q87" s="5" t="inlineStr"/>
-      <c r="R87" s="5" t="inlineStr"/>
-      <c r="S87" s="6" t="inlineStr"/>
+      <c r="Q87" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R87" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S87" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T87" s="4" t="inlineStr"/>
     </row>
     <row r="88" ht="110" customHeight="1">
@@ -7521,9 +8485,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q88" s="5" t="inlineStr"/>
-      <c r="R88" s="5" t="inlineStr"/>
-      <c r="S88" s="6" t="inlineStr"/>
+      <c r="Q88" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R88" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S88" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T88" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -7603,9 +8579,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q89" s="5" t="inlineStr"/>
-      <c r="R89" s="5" t="inlineStr"/>
-      <c r="S89" s="6" t="inlineStr"/>
+      <c r="Q89" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R89" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S89" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T89" s="4" t="inlineStr"/>
     </row>
     <row r="90" ht="110" customHeight="1">
@@ -7681,9 +8669,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q90" s="5" t="inlineStr"/>
-      <c r="R90" s="5" t="inlineStr"/>
-      <c r="S90" s="6" t="inlineStr"/>
+      <c r="Q90" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R90" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S90" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T90" s="4" t="inlineStr"/>
     </row>
     <row r="91" ht="110" customHeight="1">
@@ -7763,9 +8763,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q91" s="5" t="inlineStr"/>
-      <c r="R91" s="5" t="inlineStr"/>
-      <c r="S91" s="6" t="inlineStr"/>
+      <c r="Q91" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R91" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S91" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T91" s="4" t="inlineStr"/>
     </row>
     <row r="92" ht="110" customHeight="1">
@@ -7841,9 +8853,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q92" s="5" t="inlineStr"/>
-      <c r="R92" s="5" t="inlineStr"/>
-      <c r="S92" s="6" t="inlineStr"/>
+      <c r="Q92" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R92" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S92" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T92" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -7927,9 +8951,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q93" s="5" t="inlineStr"/>
-      <c r="R93" s="5" t="inlineStr"/>
-      <c r="S93" s="6" t="inlineStr"/>
+      <c r="Q93" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R93" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S93" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T93" s="4" t="inlineStr"/>
     </row>
     <row r="94" ht="110" customHeight="1">
@@ -8005,9 +9041,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q94" s="5" t="inlineStr"/>
-      <c r="R94" s="5" t="inlineStr"/>
-      <c r="S94" s="6" t="inlineStr"/>
+      <c r="Q94" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R94" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S94" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: lokasi POHON menjadi ?. Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T94" s="4" t="inlineStr"/>
     </row>
     <row r="95" ht="110" customHeight="1">
@@ -8087,9 +9135,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q95" s="5" t="inlineStr"/>
-      <c r="R95" s="5" t="inlineStr"/>
-      <c r="S95" s="6" t="inlineStr"/>
+      <c r="Q95" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R95" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S95" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T95" s="4" t="inlineStr"/>
     </row>
     <row r="96" ht="110" customHeight="1">
@@ -8165,9 +9225,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q96" s="5" t="inlineStr"/>
-      <c r="R96" s="5" t="inlineStr"/>
-      <c r="S96" s="6" t="inlineStr"/>
+      <c r="Q96" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R96" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S96" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: lokasi POHON menjadi ?. Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T96" s="4" t="inlineStr"/>
     </row>
     <row r="97" ht="110" customHeight="1">
@@ -8247,9 +9319,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q97" s="5" t="inlineStr"/>
-      <c r="R97" s="5" t="inlineStr"/>
-      <c r="S97" s="6" t="inlineStr"/>
+      <c r="Q97" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R97" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S97" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T97" s="4" t="inlineStr"/>
     </row>
     <row r="98" ht="110" customHeight="1">
@@ -8329,9 +9413,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q98" s="5" t="inlineStr"/>
-      <c r="R98" s="5" t="inlineStr"/>
-      <c r="S98" s="6" t="inlineStr"/>
+      <c r="Q98" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R98" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S98" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T98" s="4" t="inlineStr"/>
     </row>
     <row r="99" ht="110" customHeight="1">
@@ -8411,9 +9507,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q99" s="5" t="inlineStr"/>
-      <c r="R99" s="5" t="inlineStr"/>
-      <c r="S99" s="6" t="inlineStr"/>
+      <c r="Q99" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R99" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S99" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T99" s="4" t="inlineStr"/>
     </row>
     <row r="100" ht="110" customHeight="1">
@@ -8493,9 +9601,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q100" s="5" t="inlineStr"/>
-      <c r="R100" s="5" t="inlineStr"/>
-      <c r="S100" s="6" t="inlineStr"/>
+      <c r="Q100" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R100" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S100" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T100" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -8575,9 +9695,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q101" s="5" t="inlineStr"/>
-      <c r="R101" s="5" t="inlineStr"/>
-      <c r="S101" s="6" t="inlineStr"/>
+      <c r="Q101" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R101" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S101" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: lokasi POHON menjadi ?. Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T101" s="4" t="inlineStr"/>
     </row>
     <row r="102" ht="110" customHeight="1">
@@ -8653,9 +9785,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q102" s="5" t="inlineStr"/>
-      <c r="R102" s="5" t="inlineStr"/>
-      <c r="S102" s="6" t="inlineStr"/>
+      <c r="Q102" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R102" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S102" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: per_kelas N menjadi Y. Kolom yang tidak pasti menurut penilai: per_kelas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T102" s="4" t="inlineStr"/>
     </row>
     <row r="103" ht="110" customHeight="1">
@@ -8731,9 +9875,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q103" s="5" t="inlineStr"/>
-      <c r="R103" s="5" t="inlineStr"/>
-      <c r="S103" s="6" t="inlineStr"/>
+      <c r="Q103" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R103" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S103" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T103" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -8813,9 +9969,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q104" s="5" t="inlineStr"/>
-      <c r="R104" s="5" t="inlineStr"/>
-      <c r="S104" s="6" t="inlineStr"/>
+      <c r="Q104" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R104" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S104" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: lokasi PABRIK menjadi POHON. Kolom yang tidak pasti menurut penilai: multipandang,lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T104" s="4" t="inlineStr"/>
     </row>
     <row r="105" ht="110" customHeight="1">
@@ -8895,9 +10063,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q105" s="5" t="inlineStr"/>
-      <c r="R105" s="5" t="inlineStr"/>
-      <c r="S105" s="6" t="inlineStr"/>
+      <c r="Q105" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R105" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S105" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T105" s="4" t="inlineStr"/>
     </row>
     <row r="106" ht="110" customHeight="1">
@@ -8973,9 +10153,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q106" s="5" t="inlineStr"/>
-      <c r="R106" s="5" t="inlineStr"/>
-      <c r="S106" s="6" t="inlineStr"/>
+      <c r="Q106" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R106" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S106" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T106" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -9055,9 +10247,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q107" s="5" t="inlineStr"/>
-      <c r="R107" s="5" t="inlineStr"/>
-      <c r="S107" s="6" t="inlineStr"/>
+      <c r="Q107" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R107" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S107" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T107" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -9137,9 +10341,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q108" s="5" t="inlineStr"/>
-      <c r="R108" s="5" t="inlineStr"/>
-      <c r="S108" s="6" t="inlineStr"/>
+      <c r="Q108" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R108" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S108" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T108" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -9219,9 +10435,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q109" s="5" t="inlineStr"/>
-      <c r="R109" s="5" t="inlineStr"/>
-      <c r="S109" s="6" t="inlineStr"/>
+      <c r="Q109" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R109" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S109" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T109" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -9305,9 +10533,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q110" s="5" t="inlineStr"/>
-      <c r="R110" s="5" t="inlineStr"/>
-      <c r="S110" s="6" t="inlineStr"/>
+      <c r="Q110" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R110" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S110" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T110" s="4" t="inlineStr"/>
     </row>
     <row r="111" ht="110" customHeight="1">
@@ -9387,9 +10627,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q111" s="5" t="inlineStr"/>
-      <c r="R111" s="5" t="inlineStr"/>
-      <c r="S111" s="6" t="inlineStr"/>
+      <c r="Q111" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R111" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S111" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T111" s="4" t="inlineStr"/>
     </row>
     <row r="112" ht="110" customHeight="1">
@@ -9469,9 +10721,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q112" s="5" t="inlineStr"/>
-      <c r="R112" s="5" t="inlineStr"/>
-      <c r="S112" s="6" t="inlineStr"/>
+      <c r="Q112" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R112" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S112" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T112" s="4" t="inlineStr"/>
     </row>
     <row r="113" ht="110" customHeight="1">
@@ -9551,9 +10815,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q113" s="5" t="inlineStr"/>
-      <c r="R113" s="5" t="inlineStr"/>
-      <c r="S113" s="6" t="inlineStr"/>
+      <c r="Q113" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R113" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S113" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T113" s="4" t="inlineStr"/>
     </row>
     <row r="114" ht="110" customHeight="1">
@@ -9633,9 +10909,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q114" s="5" t="inlineStr"/>
-      <c r="R114" s="5" t="inlineStr"/>
-      <c r="S114" s="6" t="inlineStr"/>
+      <c r="Q114" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R114" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S114" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T114" s="4" t="inlineStr"/>
     </row>
     <row r="115" ht="110" customHeight="1">
@@ -9711,9 +10999,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q115" s="5" t="inlineStr"/>
+      <c r="Q115" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="R115" s="5" t="inlineStr"/>
-      <c r="S115" s="6" t="inlineStr"/>
+      <c r="S115" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Penilai dan pemeriksa berbeda: lokasi PABRIK lawan ?. Kolom yang tidak pasti menurut penilai: lokasi,tugas. Penilaian ulang Sonnet 5.5, 13 Oktober 2026, dari abstrak: C3; kode rinci berbeda dari kode lembar (tugas LF lawan KLS; lokasi TANAH lawan ?), belum diperiksa agen kedua. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T115" s="4" t="inlineStr"/>
     </row>
     <row r="116" ht="110" customHeight="1">
@@ -9789,9 +11085,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q116" s="5" t="inlineStr"/>
-      <c r="R116" s="5" t="inlineStr"/>
-      <c r="S116" s="6" t="inlineStr"/>
+      <c r="Q116" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R116" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S116" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T116" s="4" t="inlineStr"/>
     </row>
     <row r="117" ht="110" customHeight="1">
@@ -9871,9 +11179,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q117" s="5" t="inlineStr"/>
+      <c r="Q117" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="R117" s="5" t="inlineStr"/>
-      <c r="S117" s="6" t="inlineStr"/>
+      <c r="S117" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: teks lengkap. Bukan C3; usul kode C1. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T117" s="4" t="inlineStr"/>
     </row>
     <row r="118" ht="110" customHeight="1">
@@ -9949,9 +11265,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q118" s="5" t="inlineStr"/>
-      <c r="R118" s="5" t="inlineStr"/>
-      <c r="S118" s="6" t="inlineStr"/>
+      <c r="Q118" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R118" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S118" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: modalitas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T118" s="4" t="inlineStr"/>
     </row>
     <row r="119" ht="110" customHeight="1">
@@ -10027,9 +11355,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q119" s="5" t="inlineStr"/>
-      <c r="R119" s="5" t="inlineStr"/>
-      <c r="S119" s="6" t="inlineStr"/>
+      <c r="Q119" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R119" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S119" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T119" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -10109,9 +11449,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q120" s="5" t="inlineStr"/>
-      <c r="R120" s="5" t="inlineStr"/>
-      <c r="S120" s="6" t="inlineStr"/>
+      <c r="Q120" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R120" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S120" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T120" s="4" t="inlineStr"/>
     </row>
     <row r="121" ht="110" customHeight="1">
@@ -10187,9 +11539,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q121" s="5" t="inlineStr"/>
-      <c r="R121" s="5" t="inlineStr"/>
-      <c r="S121" s="6" t="inlineStr"/>
+      <c r="Q121" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R121" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S121" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T121" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -10269,9 +11633,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q122" s="5" t="inlineStr"/>
-      <c r="R122" s="5" t="inlineStr"/>
-      <c r="S122" s="6" t="inlineStr"/>
+      <c r="Q122" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R122" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S122" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T122" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -10351,9 +11727,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q123" s="5" t="inlineStr"/>
-      <c r="R123" s="5" t="inlineStr"/>
-      <c r="S123" s="6" t="inlineStr"/>
+      <c r="Q123" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R123" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S123" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T123" s="4" t="inlineStr"/>
     </row>
     <row r="124" ht="110" customHeight="1">
@@ -10429,9 +11817,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q124" s="5" t="inlineStr"/>
-      <c r="R124" s="5" t="inlineStr"/>
-      <c r="S124" s="6" t="inlineStr"/>
+      <c r="Q124" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R124" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S124" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: modalitas MSI menjadi HSI. Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T124" s="4" t="inlineStr"/>
     </row>
     <row r="125" ht="110" customHeight="1">
@@ -10507,9 +11907,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q125" s="5" t="inlineStr"/>
-      <c r="R125" s="5" t="inlineStr"/>
-      <c r="S125" s="6" t="inlineStr"/>
+      <c r="Q125" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R125" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S125" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: lokasi POHON menjadi ?. Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T125" s="4" t="inlineStr"/>
     </row>
     <row r="126" ht="110" customHeight="1">
@@ -10589,9 +12001,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q126" s="5" t="inlineStr"/>
-      <c r="R126" s="5" t="inlineStr"/>
-      <c r="S126" s="6" t="inlineStr"/>
+      <c r="Q126" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R126" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S126" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T126" s="4" t="inlineStr"/>
     </row>
     <row r="127" ht="110" customHeight="1">
@@ -10671,9 +12095,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q127" s="5" t="inlineStr"/>
+      <c r="Q127" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="R127" s="5" t="inlineStr"/>
-      <c r="S127" s="6" t="inlineStr"/>
+      <c r="S127" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: teks lengkap. Bukan C3; usul kode C1. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T127" s="4" t="inlineStr"/>
     </row>
     <row r="128" ht="110" customHeight="1">
@@ -10749,9 +12181,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q128" s="5" t="inlineStr"/>
-      <c r="R128" s="5" t="inlineStr"/>
-      <c r="S128" s="6" t="inlineStr"/>
+      <c r="Q128" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R128" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S128" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T128" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -10835,9 +12279,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q129" s="5" t="inlineStr"/>
-      <c r="R129" s="5" t="inlineStr"/>
-      <c r="S129" s="6" t="inlineStr"/>
+      <c r="Q129" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R129" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S129" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T129" s="4" t="inlineStr"/>
     </row>
     <row r="130" ht="110" customHeight="1">
@@ -10913,9 +12369,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q130" s="5" t="inlineStr"/>
-      <c r="R130" s="5" t="inlineStr"/>
-      <c r="S130" s="6" t="inlineStr"/>
+      <c r="Q130" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R130" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S130" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T130" s="4" t="inlineStr"/>
     </row>
     <row r="131" ht="110" customHeight="1">
@@ -10991,9 +12459,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q131" s="5" t="inlineStr"/>
-      <c r="R131" s="5" t="inlineStr"/>
-      <c r="S131" s="6" t="inlineStr"/>
+      <c r="Q131" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R131" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S131" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T131" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -11073,9 +12553,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q132" s="5" t="inlineStr"/>
+      <c r="Q132" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="R132" s="5" t="inlineStr"/>
-      <c r="S132" s="6" t="inlineStr"/>
+      <c r="S132" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Bukti tidak cukup untuk memutuskan (tebakan: C3). Penilaian ulang Sonnet 5.5, 13 Oktober 2026, dari abstrak: C3; kode rinci berbeda dari kode lembar (tugas SENSOR lawan KLS; lokasi POHON lawan ?), belum diperiksa agen kedua. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T132" s="4" t="inlineStr"/>
     </row>
     <row r="133" ht="110" customHeight="1">
@@ -11151,9 +12639,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q133" s="5" t="inlineStr"/>
+      <c r="Q133" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="R133" s="5" t="inlineStr"/>
-      <c r="S133" s="6" t="inlineStr"/>
+      <c r="S133" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Penilai dan pemeriksa berbeda: lokasi POHON lawan ?. Kolom yang tidak pasti menurut penilai: lokasi,per_kelas. Penilaian ulang Sonnet 5.5, 13 Oktober 2026, dari abstrak: C3; kode rinci berbeda dari kode lembar (lokasi POHON lawan ?), belum diperiksa agen kedua. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T133" s="4" t="inlineStr"/>
     </row>
     <row r="134" ht="110" customHeight="1">
@@ -11233,9 +12729,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q134" s="5" t="inlineStr"/>
-      <c r="R134" s="5" t="inlineStr"/>
-      <c r="S134" s="6" t="inlineStr"/>
+      <c r="Q134" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R134" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S134" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T134" s="4" t="inlineStr"/>
     </row>
     <row r="135" ht="110" customHeight="1">
@@ -11311,9 +12819,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q135" s="5" t="inlineStr"/>
-      <c r="R135" s="5" t="inlineStr"/>
-      <c r="S135" s="6" t="inlineStr"/>
+      <c r="Q135" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R135" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S135" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: lokasi POHON menjadi ?. Kolom yang tidak pasti menurut penilai: lokasi,modalitas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T135" s="4" t="inlineStr"/>
     </row>
     <row r="136" ht="110" customHeight="1">
@@ -11389,9 +12909,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q136" s="5" t="inlineStr"/>
-      <c r="R136" s="5" t="inlineStr"/>
-      <c r="S136" s="6" t="inlineStr"/>
+      <c r="Q136" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R136" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S136" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T136" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -11475,9 +13007,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q137" s="5" t="inlineStr"/>
-      <c r="R137" s="5" t="inlineStr"/>
-      <c r="S137" s="6" t="inlineStr"/>
+      <c r="Q137" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R137" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S137" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: teks lengkap.  Kolom yang tidak pasti menurut penilai: multipandang. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T137" s="4" t="inlineStr"/>
     </row>
     <row r="138" ht="110" customHeight="1">
@@ -11553,9 +13097,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q138" s="5" t="inlineStr"/>
-      <c r="R138" s="5" t="inlineStr"/>
-      <c r="S138" s="6" t="inlineStr"/>
+      <c r="Q138" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R138" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S138" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T138" s="4" t="inlineStr"/>
     </row>
     <row r="139" ht="110" customHeight="1">
@@ -11631,9 +13187,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q139" s="5" t="inlineStr"/>
-      <c r="R139" s="5" t="inlineStr"/>
-      <c r="S139" s="6" t="inlineStr"/>
+      <c r="Q139" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R139" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S139" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T139" s="4" t="inlineStr"/>
     </row>
     <row r="140" ht="110" customHeight="1">
@@ -11713,9 +13281,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q140" s="5" t="inlineStr"/>
-      <c r="R140" s="5" t="inlineStr"/>
-      <c r="S140" s="6" t="inlineStr"/>
+      <c r="Q140" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R140" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S140" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T140" s="4" t="inlineStr"/>
     </row>
     <row r="141" ht="110" customHeight="1">
@@ -11791,9 +13371,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q141" s="5" t="inlineStr"/>
-      <c r="R141" s="5" t="inlineStr"/>
-      <c r="S141" s="6" t="inlineStr"/>
+      <c r="Q141" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R141" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S141" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi,modalitas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T141" s="4" t="inlineStr"/>
     </row>
     <row r="142" ht="110" customHeight="1">
@@ -11869,9 +13461,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q142" s="5" t="inlineStr"/>
-      <c r="R142" s="5" t="inlineStr"/>
-      <c r="S142" s="6" t="inlineStr"/>
+      <c r="Q142" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R142" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S142" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: lokasi ? menjadi PABRIK. Kolom yang tidak pasti menurut penilai: lokasi,tugas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T142" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -11951,9 +13555,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q143" s="5" t="inlineStr"/>
-      <c r="R143" s="5" t="inlineStr"/>
-      <c r="S143" s="6" t="inlineStr"/>
+      <c r="Q143" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R143" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S143" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T143" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -12033,9 +13649,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q144" s="5" t="inlineStr"/>
-      <c r="R144" s="5" t="inlineStr"/>
-      <c r="S144" s="6" t="inlineStr"/>
+      <c r="Q144" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R144" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S144" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: tugas,lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T144" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -12115,9 +13743,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q145" s="5" t="inlineStr"/>
-      <c r="R145" s="5" t="inlineStr"/>
-      <c r="S145" s="6" t="inlineStr"/>
+      <c r="Q145" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R145" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S145" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T145" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -12197,9 +13837,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q146" s="5" t="inlineStr"/>
-      <c r="R146" s="5" t="inlineStr"/>
-      <c r="S146" s="6" t="inlineStr"/>
+      <c r="Q146" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R146" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S146" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T146" s="4" t="inlineStr"/>
     </row>
     <row r="147" ht="110" customHeight="1">
@@ -12279,9 +13931,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q147" s="5" t="inlineStr"/>
-      <c r="R147" s="5" t="inlineStr"/>
-      <c r="S147" s="6" t="inlineStr"/>
+      <c r="Q147" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R147" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S147" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T147" s="4" t="inlineStr"/>
     </row>
     <row r="148" ht="110" customHeight="1">
@@ -12357,9 +14021,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q148" s="5" t="inlineStr"/>
-      <c r="R148" s="5" t="inlineStr"/>
-      <c r="S148" s="6" t="inlineStr"/>
+      <c r="Q148" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R148" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S148" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T148" s="4" t="inlineStr"/>
     </row>
     <row r="149" ht="110" customHeight="1">
@@ -12435,9 +14111,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q149" s="5" t="inlineStr"/>
-      <c r="R149" s="5" t="inlineStr"/>
-      <c r="S149" s="6" t="inlineStr"/>
+      <c r="Q149" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R149" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S149" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T149" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -12517,9 +14205,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q150" s="5" t="inlineStr"/>
-      <c r="R150" s="5" t="inlineStr"/>
-      <c r="S150" s="6" t="inlineStr"/>
+      <c r="Q150" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R150" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S150" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T150" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -12599,9 +14299,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q151" s="5" t="inlineStr"/>
-      <c r="R151" s="5" t="inlineStr"/>
-      <c r="S151" s="6" t="inlineStr"/>
+      <c r="Q151" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R151" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S151" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: tugas SENSOR menjadi KLS; modalitas MSI menjadi RGB. Kolom yang tidak pasti menurut penilai: lokasi,modalitas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T151" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -12681,9 +14393,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q152" s="5" t="inlineStr"/>
-      <c r="R152" s="5" t="inlineStr"/>
-      <c r="S152" s="6" t="inlineStr"/>
+      <c r="Q152" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R152" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S152" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T152" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -12763,9 +14487,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q153" s="5" t="inlineStr"/>
-      <c r="R153" s="5" t="inlineStr"/>
-      <c r="S153" s="6" t="inlineStr"/>
+      <c r="Q153" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R153" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S153" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T153" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -12849,9 +14585,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q154" s="5" t="inlineStr"/>
-      <c r="R154" s="5" t="inlineStr"/>
-      <c r="S154" s="6" t="inlineStr"/>
+      <c r="Q154" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R154" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S154" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T154" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -12935,9 +14683,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q155" s="5" t="inlineStr"/>
-      <c r="R155" s="5" t="inlineStr"/>
-      <c r="S155" s="6" t="inlineStr"/>
+      <c r="Q155" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R155" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S155" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T155" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -13021,9 +14781,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q156" s="5" t="inlineStr"/>
-      <c r="R156" s="5" t="inlineStr"/>
-      <c r="S156" s="6" t="inlineStr"/>
+      <c r="Q156" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R156" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S156" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T156" s="4" t="inlineStr"/>
     </row>
     <row r="157" ht="110" customHeight="1">
@@ -13099,9 +14871,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q157" s="5" t="inlineStr"/>
-      <c r="R157" s="5" t="inlineStr"/>
-      <c r="S157" s="6" t="inlineStr"/>
+      <c r="Q157" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R157" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S157" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T157" s="4" t="inlineStr"/>
     </row>
     <row r="158" ht="110" customHeight="1">
@@ -13177,9 +14961,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q158" s="5" t="inlineStr"/>
-      <c r="R158" s="5" t="inlineStr"/>
-      <c r="S158" s="6" t="inlineStr"/>
+      <c r="Q158" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R158" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S158" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T158" s="4" t="inlineStr"/>
     </row>
     <row r="159" ht="110" customHeight="1">
@@ -13255,9 +15051,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q159" s="5" t="inlineStr"/>
-      <c r="R159" s="5" t="inlineStr"/>
-      <c r="S159" s="6" t="inlineStr"/>
+      <c r="Q159" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R159" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S159" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T159" s="4" t="inlineStr"/>
     </row>
     <row r="160" ht="110" customHeight="1">
@@ -13337,9 +15145,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q160" s="5" t="inlineStr"/>
-      <c r="R160" s="5" t="inlineStr"/>
-      <c r="S160" s="6" t="inlineStr"/>
+      <c r="Q160" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R160" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S160" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T160" s="4" t="inlineStr"/>
     </row>
     <row r="161" ht="110" customHeight="1">
@@ -13415,9 +15235,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q161" s="5" t="inlineStr"/>
-      <c r="R161" s="5" t="inlineStr"/>
-      <c r="S161" s="6" t="inlineStr"/>
+      <c r="Q161" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R161" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S161" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: modalitas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T161" s="4" t="inlineStr"/>
     </row>
     <row r="162" ht="110" customHeight="1">
@@ -13493,9 +15325,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q162" s="5" t="inlineStr"/>
-      <c r="R162" s="5" t="inlineStr"/>
-      <c r="S162" s="6" t="inlineStr"/>
+      <c r="Q162" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R162" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S162" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: lokasi PABRIK menjadi ?; per_kelas Y menjadi N. Kolom yang tidak pasti menurut penilai: lokasi,per_kelas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T162" s="4" t="inlineStr"/>
     </row>
     <row r="163" ht="110" customHeight="1">
@@ -13571,9 +15415,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q163" s="5" t="inlineStr"/>
-      <c r="R163" s="5" t="inlineStr"/>
-      <c r="S163" s="6" t="inlineStr"/>
+      <c r="Q163" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R163" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S163" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi,modalitas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T163" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -13653,9 +15509,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q164" s="5" t="inlineStr"/>
-      <c r="R164" s="5" t="inlineStr"/>
-      <c r="S164" s="6" t="inlineStr"/>
+      <c r="Q164" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R164" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S164" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T164" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -13739,9 +15607,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q165" s="5" t="inlineStr"/>
-      <c r="R165" s="5" t="inlineStr"/>
-      <c r="S165" s="6" t="inlineStr"/>
+      <c r="Q165" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R165" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S165" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T165" s="4" t="inlineStr"/>
     </row>
     <row r="166" ht="110" customHeight="1">
@@ -13817,9 +15697,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q166" s="5" t="inlineStr"/>
-      <c r="R166" s="5" t="inlineStr"/>
-      <c r="S166" s="6" t="inlineStr"/>
+      <c r="Q166" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R166" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S166" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: modalitas MSI menjadi NIR; per_kelas Y menjadi N. Kolom yang tidak pasti menurut penilai: lokasi,modalitas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T166" s="4" t="inlineStr"/>
     </row>
     <row r="167" ht="110" customHeight="1">
@@ -13899,9 +15791,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q167" s="5" t="inlineStr"/>
-      <c r="R167" s="5" t="inlineStr"/>
-      <c r="S167" s="6" t="inlineStr"/>
+      <c r="Q167" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R167" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S167" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T167" s="4" t="inlineStr"/>
     </row>
     <row r="168" ht="110" customHeight="1">
@@ -13977,9 +15881,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q168" s="5" t="inlineStr"/>
-      <c r="R168" s="5" t="inlineStr"/>
-      <c r="S168" s="6" t="inlineStr"/>
+      <c r="Q168" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R168" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S168" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: modalitas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T168" s="4" t="inlineStr"/>
     </row>
     <row r="169" ht="110" customHeight="1">
@@ -14059,9 +15975,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q169" s="5" t="inlineStr"/>
-      <c r="R169" s="5" t="inlineStr"/>
-      <c r="S169" s="6" t="inlineStr"/>
+      <c r="Q169" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R169" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S169" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (satu putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T169" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -14141,9 +16069,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q170" s="5" t="inlineStr"/>
-      <c r="R170" s="5" t="inlineStr"/>
-      <c r="S170" s="6" t="inlineStr"/>
+      <c r="Q170" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R170" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S170" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T170" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -14223,9 +16163,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q171" s="5" t="inlineStr"/>
-      <c r="R171" s="5" t="inlineStr"/>
-      <c r="S171" s="6" t="inlineStr"/>
+      <c r="Q171" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R171" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S171" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: konfirmasi Haiku 5.5 (dua putaran). Dikonfirmasi Haiku 5.5, 11 Oktober 2026 (cek_C3_haiku_ulang.csv). Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T171" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -14305,9 +16257,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q172" s="5" t="inlineStr"/>
-      <c r="R172" s="5" t="inlineStr"/>
-      <c r="S172" s="6" t="inlineStr"/>
+      <c r="Q172" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R172" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S172" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak.  Kolom yang tidak pasti menurut penilai: tugas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T172" s="4" t="inlineStr"/>
     </row>
     <row r="173" ht="110" customHeight="1">
@@ -14383,9 +16347,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q173" s="5" t="inlineStr"/>
-      <c r="R173" s="5" t="inlineStr"/>
-      <c r="S173" s="6" t="inlineStr"/>
+      <c r="Q173" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R173" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S173" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: tugas KLS menjadi SENSOR. Kolom yang tidak pasti menurut penilai: lokasi,modalitas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T173" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -14465,9 +16441,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q174" s="5" t="inlineStr"/>
-      <c r="R174" s="5" t="inlineStr"/>
-      <c r="S174" s="6" t="inlineStr"/>
+      <c r="Q174" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R174" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S174" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: per_kelas Y menjadi N. Kolom yang tidak pasti menurut penilai: lokasi,tugas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T174" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -14547,9 +16535,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q175" s="5" t="inlineStr"/>
-      <c r="R175" s="5" t="inlineStr"/>
-      <c r="S175" s="6" t="inlineStr"/>
+      <c r="Q175" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R175" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S175" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: lokasi ? menjadi PABRIK; per_kelas N menjadi Y. Kolom yang tidak pasti menurut penilai: tugas,lokasi. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T175" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -14629,9 +16629,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q176" s="5" t="inlineStr"/>
+      <c r="Q176" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="R176" s="5" t="inlineStr"/>
-      <c r="S176" s="6" t="inlineStr"/>
+      <c r="S176" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Penilai dan pemeriksa berbeda: modalitas RGB lawan RGB+NIR. Kolom yang tidak pasti menurut penilai: lokasi,modalitas,tugas. Penilaian ulang Sonnet 5.5, 13 Oktober 2026, dari abstrak: C3; kode rinci berbeda dari kode lembar (tugas SENSOR lawan MUTU; per_kelas N lawan Y), belum diperiksa agen kedua. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T176" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>
@@ -14711,9 +16719,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q177" s="5" t="inlineStr"/>
-      <c r="R177" s="5" t="inlineStr"/>
-      <c r="S177" s="6" t="inlineStr"/>
+      <c r="Q177" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R177" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S177" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 13 Oktober 2026 atas instruksi peninjau dari draf model (hasil-kerja-ai/menunggu-acc/cek-2/usul_isian_cek_C3.csv). Dasar: penilaian buta Opus 5.5 + verifikasi. Penilaian buta Opus 5.5 dan verifikasi ulang agen Opus 5.5 kedua, 12 Oktober 2026; sumber: abstrak. Usul koreksi kode: lokasi ? menjadi POHON. Kolom yang tidak pasti menurut penilai: tugas,multipandang,per_kelas. Belum dibaca peninjau.</t>
+        </is>
+      </c>
       <c r="T177" s="4" t="inlineStr">
         <is>
           <t>kode '?' pada: lokasi</t>

</xml_diff>